<commit_message>
Set FY2027 opening ceremony to 4/6 and entrance ceremony to 4/7
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FawjLRytv2ATkyFXeWDDqM
</commit_message>
<xml_diff>
--- a/令和9年度_年間計画（案）.xlsx
+++ b/令和9年度_年間計画（案）.xlsx
@@ -15047,7 +15047,7 @@
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7252">
+  <cellXfs count="7253">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <protection locked="0" hidden="0"/>
     </xf>
@@ -36630,9 +36630,15 @@
     <xf numFmtId="1" fontId="28" fillId="7" borderId="119" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="2">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="1" fontId="112" fillId="0" borderId="127" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="2">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="1" fontId="113" fillId="7" borderId="127" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="2">
       <alignment vertical="center" shrinkToFit="1"/>
     </xf>
+    <xf numFmtId="1" fontId="112" fillId="0" borderId="119" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="2">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="1" fontId="17" fillId="7" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="2">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -36653,9 +36659,6 @@
     </xf>
     <xf numFmtId="1" fontId="28" fillId="7" borderId="127" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="2">
       <alignment horizontal="justify" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="112" fillId="0" borderId="127" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="2">
-      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="1" fontId="113" fillId="0" borderId="127" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="2">
       <alignment horizontal="center" vertical="center"/>
@@ -38752,15 +38755,11 @@
     </row>
     <row r="12" ht="23.1" customFormat="1" customHeight="1" s="417">
       <c r="A12" s="446" t="n"/>
-      <c r="B12" s="508" t="n">
+      <c r="B12" s="7068" t="n">
         <v>5</v>
       </c>
-      <c r="C12" s="7051" t="inlineStr">
-        <is>
-          <t>着任式　始業式</t>
-        </is>
-      </c>
-      <c r="D12" s="670" t="n"/>
+      <c r="C12" s="7053" t="n"/>
+      <c r="D12" s="7074" t="n"/>
       <c r="E12" s="7071" t="n">
         <v>5</v>
       </c>
@@ -38896,13 +38895,13 @@
     </row>
     <row r="13" ht="22.5" customFormat="1" customHeight="1" s="417">
       <c r="A13" s="446" t="n"/>
-      <c r="B13" s="503" t="inlineStr">
+      <c r="B13" s="7059" t="inlineStr">
         <is>
           <t>月</t>
         </is>
       </c>
-      <c r="C13" s="516" t="n"/>
-      <c r="D13" s="520" t="n"/>
+      <c r="C13" s="7064" t="n"/>
+      <c r="D13" s="7079" t="n"/>
       <c r="E13" s="7048" t="inlineStr">
         <is>
           <t>水</t>
@@ -39041,7 +39040,7 @@
       </c>
       <c r="C14" s="7051" t="inlineStr">
         <is>
-          <t xml:space="preserve">入学式　</t>
+          <t>着任式　始業式</t>
         </is>
       </c>
       <c r="D14" s="480" t="n"/>
@@ -39333,7 +39332,7 @@
       </c>
       <c r="C16" s="7051" t="inlineStr">
         <is>
-          <t>生徒会オリエンテーション</t>
+          <t xml:space="preserve">入学式　</t>
         </is>
       </c>
       <c r="D16" s="641" t="n"/>
@@ -39498,11 +39497,7 @@
           <t>水</t>
         </is>
       </c>
-      <c r="C17" s="7056" t="inlineStr">
-        <is>
-          <t>対面式　身体測定(3年)</t>
-        </is>
-      </c>
+      <c r="C17" s="433" t="n"/>
       <c r="D17" s="520" t="n"/>
       <c r="E17" s="490" t="inlineStr">
         <is>
@@ -39657,15 +39652,14 @@
       </c>
       <c r="C18" s="7117" t="inlineStr">
         <is>
-          <t>身体測定(1年･IJ)</t>
+          <t>生徒会オリエンテーション</t>
         </is>
       </c>
       <c r="D18" s="641" t="inlineStr">
         <is>
-          <t>職2
-部会
-努･採
-運2</t>
+          <t>学3
+教
+部会</t>
         </is>
       </c>
       <c r="E18" s="7071" t="n">
@@ -39784,14 +39778,14 @@
       </c>
       <c r="C19" s="7133" t="inlineStr">
         <is>
-          <t>ノー部活デー</t>
+          <t>対面式　身体測定(3年)</t>
         </is>
       </c>
       <c r="D19" s="520" t="inlineStr">
         <is>
-          <t>学3
-教
-部会</t>
+          <t>努･採
+運2
+職2</t>
         </is>
       </c>
       <c r="E19" s="7048" t="inlineStr">
@@ -39888,7 +39882,7 @@
       </c>
       <c r="C20" s="7117" t="inlineStr">
         <is>
-          <t>身体測定(2年)</t>
+          <t>身体測定(1年･IJ)</t>
         </is>
       </c>
       <c r="D20" s="663" t="n"/>
@@ -40002,7 +39996,7 @@
       </c>
       <c r="C21" s="7133" t="inlineStr">
         <is>
-          <t>（ランチ４月スタート分〆切）</t>
+          <t>ノー部活デー</t>
         </is>
       </c>
       <c r="D21" s="454" t="n"/>
@@ -40521,9 +40515,9 @@
       <c r="B26" s="508" t="n">
         <v>12</v>
       </c>
-      <c r="C26" s="7051" t="inlineStr">
-        <is>
-          <t xml:space="preserve">学級写真撮影　</t>
+      <c r="C26" s="7161" t="inlineStr">
+        <is>
+          <t>※身体測定(2年)</t>
         </is>
       </c>
       <c r="D26" s="670" t="n"/>
@@ -40543,7 +40537,7 @@
       <c r="H26" s="7071" t="n">
         <v>12</v>
       </c>
-      <c r="I26" s="7161" t="inlineStr">
+      <c r="I26" s="7162" t="inlineStr">
         <is>
           <t xml:space="preserve">　 </t>
         </is>
@@ -40633,9 +40627,9 @@
           <t>月</t>
         </is>
       </c>
-      <c r="C27" s="7056" t="inlineStr">
-        <is>
-          <t xml:space="preserve">部活紹介　</t>
+      <c r="C27" s="7163" t="inlineStr">
+        <is>
+          <t xml:space="preserve">※（ランチ４月スタート分〆切）・学級写真撮影　・部活紹介　</t>
         </is>
       </c>
       <c r="D27" s="520" t="n"/>
@@ -40651,7 +40645,7 @@
           <t>土</t>
         </is>
       </c>
-      <c r="I27" s="7162" t="n"/>
+      <c r="I27" s="7164" t="n"/>
       <c r="J27" s="7065" t="n"/>
       <c r="K27" s="503" t="inlineStr">
         <is>
@@ -40720,13 +40714,13 @@
         </is>
       </c>
       <c r="AG27" s="7060" t="n"/>
-      <c r="AH27" s="7163" t="n"/>
+      <c r="AH27" s="7165" t="n"/>
       <c r="AI27" s="7048" t="inlineStr">
         <is>
           <t>日</t>
         </is>
       </c>
-      <c r="AJ27" s="7164" t="n"/>
+      <c r="AJ27" s="7166" t="n"/>
       <c r="AK27" s="7100" t="n"/>
       <c r="AL27" s="446" t="n"/>
       <c r="AM27" s="447" t="n"/>
@@ -40752,7 +40746,7 @@
           <t>学5</t>
         </is>
       </c>
-      <c r="H28" s="7165" t="n">
+      <c r="H28" s="7167" t="n">
         <v>13</v>
       </c>
       <c r="I28" s="7089" t="n"/>
@@ -40858,7 +40852,7 @@
           <t>職4</t>
         </is>
       </c>
-      <c r="H29" s="7166" t="inlineStr">
+      <c r="H29" s="7168" t="inlineStr">
         <is>
           <t>日</t>
         </is>
@@ -40920,7 +40914,7 @@
           <t>木</t>
         </is>
       </c>
-      <c r="AD29" s="7167" t="inlineStr">
+      <c r="AD29" s="7169" t="inlineStr">
         <is>
           <t>｜</t>
         </is>
@@ -40976,7 +40970,7 @@
       <c r="N30" s="7071" t="n">
         <v>14</v>
       </c>
-      <c r="O30" s="7168" t="n"/>
+      <c r="O30" s="7170" t="n"/>
       <c r="P30" s="7092" t="n"/>
       <c r="Q30" s="474" t="n">
         <v>14</v>
@@ -41026,7 +41020,7 @@
       <c r="AF30" s="474" t="n">
         <v>14</v>
       </c>
-      <c r="AG30" s="7169" t="inlineStr">
+      <c r="AG30" s="7161" t="inlineStr">
         <is>
           <t>※↓【定時制１次入試】</t>
         </is>
@@ -41039,7 +41033,7 @@
       <c r="AI30" s="474" t="n">
         <v>14</v>
       </c>
-      <c r="AJ30" s="7170" t="inlineStr">
+      <c r="AJ30" s="7171" t="inlineStr">
         <is>
           <t>R7生徒会オリ(リハ)</t>
         </is>
@@ -41165,7 +41159,8 @@
         <is>
           <t>職3
 現1
-定</t>
+定
+部会</t>
         </is>
       </c>
       <c r="E32" s="7071" t="n">
@@ -41284,8 +41279,8 @@
           <t>土</t>
         </is>
       </c>
-      <c r="F33" s="7171" t="n"/>
-      <c r="G33" s="7172" t="n"/>
+      <c r="F33" s="7172" t="n"/>
+      <c r="G33" s="7173" t="n"/>
       <c r="H33" s="503" t="inlineStr">
         <is>
           <t>火</t>
@@ -41391,7 +41386,7 @@
       <c r="H34" s="474" t="n">
         <v>16</v>
       </c>
-      <c r="I34" s="7173" t="inlineStr">
+      <c r="I34" s="7174" t="inlineStr">
         <is>
           <t>｜│</t>
         </is>
@@ -41503,7 +41498,7 @@
           <t>水</t>
         </is>
       </c>
-      <c r="I35" s="7174" t="inlineStr">
+      <c r="I35" s="7175" t="inlineStr">
         <is>
           <t>↓↓</t>
         </is>
@@ -41579,13 +41574,13 @@
           <t>水</t>
         </is>
       </c>
-      <c r="AG35" s="7175" t="n"/>
+      <c r="AG35" s="7176" t="n"/>
       <c r="AI35" s="490" t="inlineStr">
         <is>
           <t>木</t>
         </is>
       </c>
-      <c r="AJ35" s="7176" t="n"/>
+      <c r="AJ35" s="7177" t="n"/>
       <c r="AK35" t="inlineStr">
         <is>
           <t>採</t>
@@ -41601,7 +41596,7 @@
         <v>17</v>
       </c>
       <c r="C36" s="7143" t="n"/>
-      <c r="D36" s="7177" t="n"/>
+      <c r="D36" s="7178" t="n"/>
       <c r="E36" s="508" t="n">
         <v>17</v>
       </c>
@@ -41679,7 +41674,7 @@
       <c r="AF36" s="474" t="n">
         <v>17</v>
       </c>
-      <c r="AG36" s="7178" t="inlineStr">
+      <c r="AG36" s="7179" t="inlineStr">
         <is>
           <t>学年保護者会(1年)</t>
         </is>
@@ -41763,7 +41758,7 @@
           <t>水</t>
         </is>
       </c>
-      <c r="X37" s="7179" t="inlineStr">
+      <c r="X37" s="7180" t="inlineStr">
         <is>
           <t>↓</t>
         </is>
@@ -41803,7 +41798,7 @@
           <t>金</t>
         </is>
       </c>
-      <c r="AJ37" s="7176" t="n"/>
+      <c r="AJ37" s="7177" t="n"/>
       <c r="AL37" s="446" t="n"/>
       <c r="AM37" s="447" t="n"/>
       <c r="BA37" s="417" t="n"/>
@@ -41818,7 +41813,7 @@
       <c r="E38" s="508" t="n">
         <v>18</v>
       </c>
-      <c r="F38" s="7180" t="inlineStr">
+      <c r="F38" s="7181" t="inlineStr">
         <is>
           <t>①確認テスト</t>
         </is>
@@ -41854,7 +41849,7 @@
       <c r="Q38" s="7068" t="n">
         <v>18</v>
       </c>
-      <c r="R38" s="7181" t="n"/>
+      <c r="R38" s="7182" t="n"/>
       <c r="S38" s="7094" t="n"/>
       <c r="T38" s="508" t="n">
         <v>18</v>
@@ -42018,7 +42013,7 @@
       <c r="E40" s="474" t="n">
         <v>19</v>
       </c>
-      <c r="F40" s="7182" t="inlineStr">
+      <c r="F40" s="7183" t="inlineStr">
         <is>
           <t>①確認テスト</t>
         </is>
@@ -42028,7 +42023,7 @@
         <v>19</v>
       </c>
       <c r="I40" s="7083" t="n"/>
-      <c r="J40" s="7183" t="n"/>
+      <c r="J40" s="7184" t="n"/>
       <c r="K40" s="7071" t="n">
         <v>19</v>
       </c>
@@ -42135,8 +42130,8 @@
           <t>土</t>
         </is>
       </c>
-      <c r="I41" s="7162" t="n"/>
-      <c r="J41" s="7184" t="n"/>
+      <c r="I41" s="7164" t="n"/>
+      <c r="J41" s="7185" t="n"/>
       <c r="K41" s="7048" t="inlineStr">
         <is>
           <t>月</t>
@@ -42150,7 +42145,7 @@
         </is>
       </c>
       <c r="O41" s="7060" t="n"/>
-      <c r="P41" s="7185" t="n"/>
+      <c r="P41" s="7186" t="n"/>
       <c r="Q41" s="7059" t="inlineStr">
         <is>
           <t>日</t>
@@ -42199,14 +42194,14 @@
           <t>土</t>
         </is>
       </c>
-      <c r="AG41" s="7186" t="n"/>
+      <c r="AG41" s="7187" t="n"/>
       <c r="AH41" s="7088" t="n"/>
       <c r="AI41" s="7048" t="inlineStr">
         <is>
           <t>日</t>
         </is>
       </c>
-      <c r="AJ41" s="7187" t="n"/>
+      <c r="AJ41" s="7188" t="n"/>
       <c r="AK41" s="7050" t="n"/>
       <c r="AL41" s="446" t="n"/>
       <c r="AM41" s="447" t="n"/>
@@ -42261,8 +42256,8 @@
       <c r="N42" s="7071" t="n">
         <v>20</v>
       </c>
-      <c r="O42" s="7188" t="n"/>
-      <c r="P42" s="7189" t="n"/>
+      <c r="O42" s="7189" t="n"/>
+      <c r="P42" s="7190" t="n"/>
       <c r="Q42" s="7068" t="n">
         <v>20</v>
       </c>
@@ -42358,14 +42353,14 @@
         </is>
       </c>
       <c r="O43" s="7060" t="n"/>
-      <c r="P43" s="7185" t="n"/>
+      <c r="P43" s="7186" t="n"/>
       <c r="Q43" s="7059" t="inlineStr">
         <is>
           <t>月</t>
         </is>
       </c>
       <c r="R43" s="7087" t="n"/>
-      <c r="S43" s="7190" t="n"/>
+      <c r="S43" s="7191" t="n"/>
       <c r="T43" s="503" t="inlineStr">
         <is>
           <t>水</t>
@@ -42379,7 +42374,7 @@
         </is>
       </c>
       <c r="X43" s="7089" t="n"/>
-      <c r="Y43" s="7191" t="n"/>
+      <c r="Y43" s="7192" t="n"/>
       <c r="Z43" s="503" t="inlineStr">
         <is>
           <t>月</t>
@@ -42449,8 +42444,8 @@
       <c r="N44" s="7071" t="n">
         <v>21</v>
       </c>
-      <c r="O44" s="7192" t="n"/>
-      <c r="P44" s="7189" t="n"/>
+      <c r="O44" s="7193" t="n"/>
+      <c r="P44" s="7190" t="n"/>
       <c r="Q44" s="508" t="n">
         <v>21</v>
       </c>
@@ -42459,7 +42454,7 @@
           <t>※ノー部活ウィーク</t>
         </is>
       </c>
-      <c r="S44" s="7193" t="n"/>
+      <c r="S44" s="7194" t="n"/>
       <c r="T44" s="508" t="n">
         <v>21</v>
       </c>
@@ -42553,7 +42548,7 @@
           <t>│</t>
         </is>
       </c>
-      <c r="S45" s="7194" t="n"/>
+      <c r="S45" s="7195" t="n"/>
       <c r="T45" s="503" t="inlineStr">
         <is>
           <t>木</t>
@@ -42642,12 +42637,12 @@
       <c r="Q46" s="508" t="n">
         <v>22</v>
       </c>
-      <c r="R46" s="7195" t="inlineStr">
+      <c r="R46" s="7196" t="inlineStr">
         <is>
           <t>│</t>
         </is>
       </c>
-      <c r="S46" s="7196" t="n"/>
+      <c r="S46" s="7197" t="n"/>
       <c r="T46" s="508" t="n">
         <v>22</v>
       </c>
@@ -42732,7 +42727,7 @@
           <t>水</t>
         </is>
       </c>
-      <c r="R47" s="7197" t="n"/>
+      <c r="R47" s="7198" t="n"/>
       <c r="S47" s="561" t="n"/>
       <c r="T47" s="503" t="inlineStr">
         <is>
@@ -42832,7 +42827,7 @@
       <c r="W48" s="7071" t="n">
         <v>23</v>
       </c>
-      <c r="X48" s="7198" t="inlineStr">
+      <c r="X48" s="7199" t="inlineStr">
         <is>
           <t>勤労感謝の日</t>
         </is>
@@ -42924,8 +42919,8 @@
           <t>木</t>
         </is>
       </c>
-      <c r="R49" s="7199" t="n"/>
-      <c r="S49" s="7200" t="n"/>
+      <c r="R49" s="7200" t="n"/>
+      <c r="S49" s="7201" t="n"/>
       <c r="T49" s="7059" t="inlineStr">
         <is>
           <t>土</t>
@@ -43101,7 +43096,7 @@
           <t>木</t>
         </is>
       </c>
-      <c r="I51" s="7201" t="inlineStr">
+      <c r="I51" s="7202" t="inlineStr">
         <is>
           <t>｜保護者試食会</t>
         </is>
@@ -43126,7 +43121,7 @@
           <t>金</t>
         </is>
       </c>
-      <c r="R51" s="7201" t="inlineStr">
+      <c r="R51" s="7202" t="inlineStr">
         <is>
           <t>│　　　　　専修合同説明会</t>
         </is>
@@ -43152,7 +43147,7 @@
         </is>
       </c>
       <c r="AA51" s="7089" t="n"/>
-      <c r="AB51" s="7202" t="n"/>
+      <c r="AB51" s="7203" t="n"/>
       <c r="AC51" s="490" t="inlineStr">
         <is>
           <t>月</t>
@@ -43165,7 +43160,7 @@
           <t>木</t>
         </is>
       </c>
-      <c r="AG51" s="7203" t="inlineStr">
+      <c r="AG51" s="7204" t="inlineStr">
         <is>
           <t>【公立一般Ａ面接】
 　　　　3年通知表(本)提出</t>
@@ -43195,7 +43190,7 @@
       <c r="B52" s="7150" t="n">
         <v>25</v>
       </c>
-      <c r="C52" s="7204" t="n"/>
+      <c r="C52" s="7205" t="n"/>
       <c r="D52" s="7070" t="n"/>
       <c r="E52" s="508" t="n">
         <v>25</v>
@@ -43274,7 +43269,7 @@
       <c r="AF52" s="474" t="n">
         <v>25</v>
       </c>
-      <c r="AG52" s="7205" t="inlineStr">
+      <c r="AG52" s="7206" t="inlineStr">
         <is>
           <t>3送会リハ①</t>
         </is>
@@ -43313,7 +43308,7 @@
           <t>金</t>
         </is>
       </c>
-      <c r="I53" s="7201" t="inlineStr">
+      <c r="I53" s="7202" t="inlineStr">
         <is>
           <t>｜</t>
         </is>
@@ -43338,12 +43333,12 @@
           <t>土</t>
         </is>
       </c>
-      <c r="R53" s="7206" t="inlineStr">
+      <c r="R53" s="7207" t="inlineStr">
         <is>
           <t>│</t>
         </is>
       </c>
-      <c r="S53" s="7200" t="n"/>
+      <c r="S53" s="7201" t="n"/>
       <c r="T53" s="503" t="inlineStr">
         <is>
           <t>月</t>
@@ -43356,7 +43351,7 @@
           <t>木</t>
         </is>
       </c>
-      <c r="X53" s="7207" t="n"/>
+      <c r="X53" s="7208" t="n"/>
       <c r="Y53" t="inlineStr">
         <is>
           <t>学10</t>
@@ -43381,7 +43376,7 @@
           <t>金</t>
         </is>
       </c>
-      <c r="AG53" s="7208" t="inlineStr">
+      <c r="AG53" s="7209" t="inlineStr">
         <is>
           <t>【公立一般Ｂ面接】</t>
         </is>
@@ -43514,7 +43509,7 @@
           <t>土</t>
         </is>
       </c>
-      <c r="I55" s="7206" t="inlineStr">
+      <c r="I55" s="7207" t="inlineStr">
         <is>
           <t>｜</t>
         </is>
@@ -43571,12 +43566,12 @@
           <t>水</t>
         </is>
       </c>
-      <c r="AD55" s="7209" t="inlineStr">
+      <c r="AD55" s="7210" t="inlineStr">
         <is>
           <t>【通信制前期合格発表】</t>
         </is>
       </c>
-      <c r="AF55" s="7210" t="inlineStr">
+      <c r="AF55" s="7211" t="inlineStr">
         <is>
           <t>土</t>
         </is>
@@ -43611,7 +43606,7 @@
       <c r="E56" s="474" t="n">
         <v>27</v>
       </c>
-      <c r="F56" s="7211" t="inlineStr">
+      <c r="F56" s="7212" t="inlineStr">
         <is>
           <t>稲武野外学習(2年)</t>
         </is>
@@ -43690,7 +43685,7 @@
         <v>27</v>
       </c>
       <c r="AJ56" s="7084" t="n"/>
-      <c r="AK56" s="7212" t="n"/>
+      <c r="AK56" s="7213" t="n"/>
       <c r="AL56" s="446" t="n"/>
       <c r="AM56" s="447" t="n"/>
     </row>
@@ -43767,7 +43762,7 @@
         </is>
       </c>
       <c r="X57" s="7112" t="n"/>
-      <c r="Y57" s="7184" t="n"/>
+      <c r="Y57" s="7185" t="n"/>
       <c r="Z57" s="7059" t="inlineStr">
         <is>
           <t>月</t>
@@ -43813,7 +43808,7 @@
       <c r="E58" s="474" t="n">
         <v>28</v>
       </c>
-      <c r="F58" s="7211" t="inlineStr">
+      <c r="F58" s="7212" t="inlineStr">
         <is>
           <t>稲武野外学習(2年)</t>
         </is>
@@ -43845,7 +43840,7 @@
       <c r="Q58" s="474" t="n">
         <v>28</v>
       </c>
-      <c r="R58" s="7213" t="inlineStr">
+      <c r="R58" s="7214" t="inlineStr">
         <is>
           <t>｜</t>
         </is>
@@ -43882,7 +43877,7 @@
       <c r="AF58" s="474" t="n">
         <v>28</v>
       </c>
-      <c r="AG58" s="7214" t="inlineStr">
+      <c r="AG58" s="7215" t="inlineStr">
         <is>
           <t>3送会準備・リハ②</t>
         </is>
@@ -43979,7 +43974,7 @@
       </c>
       <c r="AD59" s="433" t="n"/>
       <c r="AE59" s="517" t="n"/>
-      <c r="AF59" s="7215" t="inlineStr">
+      <c r="AF59" s="7216" t="inlineStr">
         <is>
           <t>月</t>
         </is>
@@ -44010,7 +44005,7 @@
       <c r="E60" s="7071" t="n">
         <v>29</v>
       </c>
-      <c r="F60" s="7216" t="n"/>
+      <c r="F60" s="7217" t="n"/>
       <c r="G60" s="7097" t="n"/>
       <c r="H60" s="508" t="n">
         <v>29</v>
@@ -44068,10 +44063,10 @@
       </c>
       <c r="AD60" s="7083" t="n"/>
       <c r="AE60" s="7079" t="n"/>
-      <c r="AF60" s="7217" t="n">
+      <c r="AF60" s="7218" t="n">
         <v>29</v>
       </c>
-      <c r="AG60" s="7218" t="inlineStr">
+      <c r="AG60" s="7219" t="inlineStr">
         <is>
           <t>3年生を送る会</t>
         </is>
@@ -44092,13 +44087,13 @@
         </is>
       </c>
       <c r="C61" s="7060" t="n"/>
-      <c r="D61" s="7219" t="n"/>
+      <c r="D61" s="7220" t="n"/>
       <c r="E61" s="7048" t="inlineStr">
         <is>
           <t>土</t>
         </is>
       </c>
-      <c r="F61" s="7220" t="n"/>
+      <c r="F61" s="7221" t="n"/>
       <c r="G61" s="7079" t="n"/>
       <c r="H61" s="503" t="inlineStr">
         <is>
@@ -44126,7 +44121,7 @@
           <t>水</t>
         </is>
       </c>
-      <c r="R61" s="7221" t="inlineStr">
+      <c r="R61" s="7222" t="inlineStr">
         <is>
           <t>生徒会･体育委員リハ</t>
         </is>
@@ -44163,7 +44158,7 @@
         </is>
       </c>
       <c r="AD61" s="7089" t="n"/>
-      <c r="AE61" s="7222" t="n"/>
+      <c r="AE61" s="7223" t="n"/>
       <c r="AF61" t="inlineStr">
         <is>
           <t>火</t>
@@ -44184,7 +44179,7 @@
       <c r="B62" s="508" t="n">
         <v>30</v>
       </c>
-      <c r="C62" s="7223" t="inlineStr">
+      <c r="C62" s="7224" t="inlineStr">
         <is>
           <t>※⑤全国学調(英話すこと）</t>
         </is>
@@ -44198,7 +44193,7 @@
         <v>30</v>
       </c>
       <c r="F62" s="7106" t="n"/>
-      <c r="G62" s="7224" t="n"/>
+      <c r="G62" s="7225" t="n"/>
       <c r="H62" s="474" t="n">
         <v>30</v>
       </c>
@@ -44239,7 +44234,7 @@
         <v>30</v>
       </c>
       <c r="U62" s="7089" t="n"/>
-      <c r="V62" s="7225" t="n"/>
+      <c r="V62" s="7226" t="n"/>
       <c r="W62" s="474" t="n">
         <v>30</v>
       </c>
@@ -44248,7 +44243,7 @@
       <c r="Z62" s="7071" t="n">
         <v>30</v>
       </c>
-      <c r="AA62" s="7226" t="inlineStr">
+      <c r="AA62" s="7227" t="inlineStr">
         <is>
           <t>｜</t>
         </is>
@@ -44263,7 +44258,7 @@
         <v>30</v>
       </c>
       <c r="AJ62" s="7053" t="n"/>
-      <c r="AK62" s="7227" t="n"/>
+      <c r="AK62" s="7228" t="n"/>
       <c r="AL62" s="446" t="n"/>
       <c r="AM62" s="447" t="n"/>
     </row>
@@ -44274,7 +44269,7 @@
           <t>金</t>
         </is>
       </c>
-      <c r="C63" s="7228" t="inlineStr">
+      <c r="C63" s="7229" t="inlineStr">
         <is>
           <t>⑤⑥修学旅行・進路説明会(3年)・部活保護者会</t>
         </is>
@@ -44299,7 +44294,7 @@
         </is>
       </c>
       <c r="L63" s="7060" t="n"/>
-      <c r="M63" s="7229" t="n"/>
+      <c r="M63" s="7230" t="n"/>
       <c r="N63" s="7059" t="inlineStr">
         <is>
           <t>月</t>
@@ -44324,7 +44319,7 @@
         </is>
       </c>
       <c r="U63" s="7112" t="n"/>
-      <c r="V63" s="7230" t="n"/>
+      <c r="V63" s="7231" t="n"/>
       <c r="W63" s="490" t="inlineStr">
         <is>
           <t>火</t>
@@ -44337,13 +44332,13 @@
           <t>木</t>
         </is>
       </c>
-      <c r="AA63" s="7231" t="inlineStr">
+      <c r="AA63" s="7232" t="inlineStr">
         <is>
           <t>｜</t>
         </is>
       </c>
-      <c r="AB63" s="7232" t="n"/>
-      <c r="AC63" s="7210" t="inlineStr">
+      <c r="AB63" s="7233" t="n"/>
+      <c r="AC63" s="7211" t="inlineStr">
         <is>
           <t>日</t>
         </is>
@@ -44356,13 +44351,13 @@
         </is>
       </c>
       <c r="AJ63" s="7060" t="n"/>
-      <c r="AK63" s="7233" t="n"/>
+      <c r="AK63" s="7234" t="n"/>
       <c r="AL63" s="446" t="n"/>
       <c r="AM63" s="447" t="n"/>
     </row>
     <row r="64" ht="23.1" customHeight="1" s="1342">
       <c r="A64" s="487" t="n"/>
-      <c r="B64" s="7234" t="n"/>
+      <c r="B64" s="7235" t="n"/>
       <c r="E64" s="474" t="n">
         <v>31</v>
       </c>
@@ -44376,28 +44371,28 @@
           <t>集</t>
         </is>
       </c>
-      <c r="H64" s="7217" t="n"/>
+      <c r="H64" s="7218" t="n"/>
       <c r="K64" s="7071" t="n">
         <v>31</v>
       </c>
       <c r="L64" s="7151" t="n"/>
-      <c r="M64" s="7235" t="n"/>
+      <c r="M64" s="7236" t="n"/>
       <c r="N64" s="7071" t="n">
         <v>31</v>
       </c>
       <c r="O64" s="7084" t="n"/>
       <c r="P64" s="7054" t="n"/>
-      <c r="Q64" s="7236" t="n"/>
+      <c r="Q64" s="7237" t="n"/>
       <c r="T64" s="7059" t="n">
         <v>31</v>
       </c>
       <c r="U64" s="7089" t="n"/>
-      <c r="V64" s="7224" t="n"/>
-      <c r="W64" s="7237" t="n"/>
+      <c r="V64" s="7225" t="n"/>
+      <c r="W64" s="7238" t="n"/>
       <c r="Z64" s="7071" t="n">
         <v>31</v>
       </c>
-      <c r="AA64" s="7226" t="inlineStr">
+      <c r="AA64" s="7227" t="inlineStr">
         <is>
           <t>ノー部活ウィーク</t>
         </is>
@@ -44415,7 +44410,7 @@
       <c r="AI64" s="7071" t="n">
         <v>31</v>
       </c>
-      <c r="AJ64" s="7188" t="n"/>
+      <c r="AJ64" s="7189" t="n"/>
       <c r="AK64" s="7100" t="n"/>
       <c r="AL64" s="471" t="n"/>
       <c r="AM64" s="447" t="n"/>
@@ -44580,54 +44575,54 @@
           <t>月</t>
         </is>
       </c>
-      <c r="F65" s="7238" t="inlineStr">
+      <c r="F65" s="7239" t="inlineStr">
         <is>
           <t>｜ノー部活ウィーク</t>
         </is>
       </c>
       <c r="G65" s="453" t="n"/>
-      <c r="K65" s="7239" t="inlineStr">
+      <c r="K65" s="7240" t="inlineStr">
         <is>
           <t>土</t>
         </is>
       </c>
-      <c r="L65" s="7240" t="n"/>
-      <c r="M65" s="7232" t="n"/>
-      <c r="N65" s="7241" t="inlineStr">
+      <c r="L65" s="7241" t="n"/>
+      <c r="M65" s="7233" t="n"/>
+      <c r="N65" s="7242" t="inlineStr">
         <is>
           <t>火</t>
         </is>
       </c>
-      <c r="O65" s="7242" t="n"/>
-      <c r="P65" s="7243" t="n"/>
-      <c r="T65" s="7244" t="inlineStr">
+      <c r="O65" s="7243" t="n"/>
+      <c r="P65" s="7244" t="n"/>
+      <c r="T65" s="7245" t="inlineStr">
         <is>
           <t>日</t>
         </is>
       </c>
-      <c r="U65" s="7245" t="n"/>
-      <c r="V65" s="7246" t="n"/>
-      <c r="Z65" s="7239" t="inlineStr">
+      <c r="U65" s="7246" t="n"/>
+      <c r="V65" s="7247" t="n"/>
+      <c r="Z65" s="7240" t="inlineStr">
         <is>
           <t>金</t>
         </is>
       </c>
-      <c r="AA65" s="7240" t="n"/>
-      <c r="AB65" s="7232" t="n"/>
+      <c r="AA65" s="7241" t="n"/>
+      <c r="AB65" s="7233" t="n"/>
       <c r="AC65" s="459" t="inlineStr">
         <is>
           <t>月</t>
         </is>
       </c>
-      <c r="AD65" s="7247" t="n"/>
+      <c r="AD65" s="7248" t="n"/>
       <c r="AE65" s="453" t="n"/>
-      <c r="AI65" s="7239" t="inlineStr">
+      <c r="AI65" s="7240" t="inlineStr">
         <is>
           <t>金</t>
         </is>
       </c>
-      <c r="AJ65" s="7240" t="n"/>
-      <c r="AK65" s="7248" t="n"/>
+      <c r="AJ65" s="7241" t="n"/>
+      <c r="AK65" s="7249" t="n"/>
       <c r="AL65" s="446" t="n"/>
       <c r="AM65" s="447" t="n"/>
     </row>
@@ -44674,30 +44669,30 @@
     </row>
     <row r="67" ht="44.25" customHeight="1" s="1342" thickBot="1">
       <c r="A67" s="446" t="n"/>
-      <c r="B67" s="7249" t="inlineStr">
+      <c r="B67" s="7250" t="inlineStr">
         <is>
           <t xml:space="preserve">　学：学年会　運：運営委員会　職：職員会議　現：現職教育　努：努力点推進員会　教支：教育支援委員会　保：学校保健委員会　進：進路指導委員会　予：予算委員会　集：集会　 　
 　採：教材採択委員会　編：学級編制会議　卒認：卒業認定会議　進認：進級認定会議　部反：年度末部会反省　全反：年度末全体反省会　委：生徒委員会　
 　議：生徒議会　教：教科部会　不：不登校生徒支援委員会　定：定時退校日　行：行事検討委員会　評：学校評議員会</t>
         </is>
       </c>
-      <c r="C67" s="7250" t="n"/>
-      <c r="D67" s="7250" t="n"/>
-      <c r="E67" s="7250" t="n"/>
-      <c r="F67" s="7250" t="n"/>
-      <c r="G67" s="7250" t="n"/>
-      <c r="H67" s="7250" t="n"/>
-      <c r="I67" s="7250" t="n"/>
-      <c r="J67" s="7250" t="n"/>
-      <c r="K67" s="7250" t="n"/>
-      <c r="L67" s="7250" t="n"/>
-      <c r="M67" s="7250" t="n"/>
-      <c r="N67" s="7250" t="n"/>
-      <c r="O67" s="7250" t="n"/>
-      <c r="P67" s="7250" t="n"/>
-      <c r="Q67" s="7250" t="n"/>
-      <c r="R67" s="7250" t="n"/>
-      <c r="S67" s="7251" t="n"/>
+      <c r="C67" s="7251" t="n"/>
+      <c r="D67" s="7251" t="n"/>
+      <c r="E67" s="7251" t="n"/>
+      <c r="F67" s="7251" t="n"/>
+      <c r="G67" s="7251" t="n"/>
+      <c r="H67" s="7251" t="n"/>
+      <c r="I67" s="7251" t="n"/>
+      <c r="J67" s="7251" t="n"/>
+      <c r="K67" s="7251" t="n"/>
+      <c r="L67" s="7251" t="n"/>
+      <c r="M67" s="7251" t="n"/>
+      <c r="N67" s="7251" t="n"/>
+      <c r="O67" s="7251" t="n"/>
+      <c r="P67" s="7251" t="n"/>
+      <c r="Q67" s="7251" t="n"/>
+      <c r="R67" s="7251" t="n"/>
+      <c r="S67" s="7252" t="n"/>
       <c r="T67" s="6116" t="inlineStr">
         <is>
           <t xml:space="preserve">講演会（時期未定）　　　　　　　
@@ -44705,29 +44700,29 @@
 　　　　　　　　　　　　　上級学校講演会（3年)　　</t>
         </is>
       </c>
-      <c r="U67" s="7250" t="n"/>
-      <c r="V67" s="7250" t="n"/>
-      <c r="W67" s="7250" t="n"/>
-      <c r="X67" s="7250" t="n"/>
-      <c r="Y67" s="7250" t="n"/>
-      <c r="Z67" s="7250" t="n"/>
-      <c r="AA67" s="7250" t="n"/>
-      <c r="AB67" s="7250" t="n"/>
+      <c r="U67" s="7251" t="n"/>
+      <c r="V67" s="7251" t="n"/>
+      <c r="W67" s="7251" t="n"/>
+      <c r="X67" s="7251" t="n"/>
+      <c r="Y67" s="7251" t="n"/>
+      <c r="Z67" s="7251" t="n"/>
+      <c r="AA67" s="7251" t="n"/>
+      <c r="AB67" s="7251" t="n"/>
       <c r="AC67" s="6118" t="inlineStr">
         <is>
           <t>２年生職場体験学習（１月）
 IJ組職場見学（１月）</t>
         </is>
       </c>
-      <c r="AD67" s="7250" t="n"/>
-      <c r="AE67" s="7250" t="n"/>
+      <c r="AD67" s="7251" t="n"/>
+      <c r="AE67" s="7251" t="n"/>
       <c r="AF67" s="6120" t="inlineStr">
         <is>
           <t xml:space="preserve">IJ組学級懇談会（２月） </t>
         </is>
       </c>
-      <c r="AG67" s="7250" t="n"/>
-      <c r="AH67" s="7250" t="n"/>
+      <c r="AG67" s="7251" t="n"/>
+      <c r="AH67" s="7251" t="n"/>
       <c r="AI67" s="445" t="inlineStr">
         <is>
           <t>IJ組校外学習（３月）</t>
@@ -45307,7 +45302,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D63"/>
+  <dimension ref="A1:D64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="1342" min="1" max="1"/>
@@ -45333,335 +45328,320 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>・日付で決まるもの（1学期終業式7/20、2学期始業式9/1、2学期終業式12/23、3学期始業式1/7、修了式3/24、夏季休業7/21〜8/31、冬季休業12/24〜1/6、学年末休業3/25〜）は日付を優先した。市の学校暦が出たら確認する。</t>
+          <t>・着任式・始業式4/6（火）、入学式4/7（水）。今年度の4/6〜4/9の行事は同じ日付に、4/10の行事は4/12に移した。</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>・祝日は令和9年度の暦で入れ直した。祝日と重なった行事は次の登校日に移し、赤字（※）で示した。</t>
+          <t>・日付で決まるもの（1学期終業式7/20、2学期始業式9/1、2学期終業式12/23、3学期始業式1/7、修了式3/24、夏季休業7/21〜8/31、冬季休業12/24〜1/6、学年末休業3/25〜）は日付を優先した。市の学校暦が出たら確認する。</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>・B帯案に合わせ、職員会議・学年会・運営委員会・現職教育・教科部会などは同じ週の木曜（研修14:05〜14:55のあと、会議15:00〜15:45）に移した。</t>
+          <t>・祝日は令和9年度の暦で入れ直した。祝日と重なった行事は次の登校日に移し、赤字（※）で示した。</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>・生徒委員会・生徒議会・集会・定時退校日・学校評議員会・提出物などは移していない。</t>
+          <t>・B帯案に合わせ、職員会議・学年会・運営委員会・現職教育・教科部会などは同じ週の木曜（研修14:05〜14:55のあと、会議15:00〜15:45）に移した。</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>・木曜の登校日は41日。体育大会・終業式など午後に研修ができない木曜を除くと35回前後で余裕が少ないため、木曜の午後には行事を入れない。</t>
+          <t>・生徒委員会・生徒議会・集会・定時退校日・学校評議員会・提出物などは移していない。</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>・保護者会・教育相談の期間（1・2年4日、3年5日）は、月行事予定・授業数カウントで反映する。</t>
+          <t>・木曜の登校日は41日。体育大会・終業式など午後に研修ができない木曜を除くと35回前後で余裕が少ないため、木曜の午後には行事を入れない。</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
+          <t>・保護者会・教育相談の期間（1・2年4日、3年5日）は、月行事予定・授業数カウントで反映する。</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
           <t>・県の入試日程、全国学力調査、修学旅行・体育大会など外部と調整する行事の日付は要確認。</t>
         </is>
       </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>要確認（祝日などと重なった行事）</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr"/>
-      <c r="C11" t="inlineStr"/>
-      <c r="D11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>元の日付</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>理由</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>行事・会議</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>対応</t>
-        </is>
-      </c>
+          <t>要確認（祝日などと重なった行事）</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr"/>
+      <c r="C12" t="inlineStr"/>
+      <c r="D12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>4/29</t>
+          <t>元の日付</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>昭和の日</t>
+          <t>理由</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>⑤全国学調(英話すこと）</t>
+          <t>行事・会議</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>4/30に移動（要調整）</t>
+          <t>対応</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>4/29</t>
+          <t>4/9</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>昭和の日</t>
+          <t>始業式を4/6にしたため</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>運4</t>
+          <t>身体測定(2年)・（ランチ４月スタート分〆切）</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>4/30に移動（会議は木曜へ移す処理あり）</t>
+          <t>4/12(月)に移動（要調整）</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>9/20</t>
+          <t>4/29</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>敬老の日</t>
+          <t>昭和の日</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>ノー部活ウィーク</t>
+          <t>⑤全国学調(英話すこと）</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>9/21に移動（要調整）</t>
+          <t>4/30に移動（要調整）</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>9/23</t>
+          <t>4/29</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>秋分の日</t>
+          <t>昭和の日</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>職8</t>
+          <t>運4</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>9/24に移動（会議は木曜へ移す処理あり）</t>
+          <t>4/30に移動（会議は木曜へ移す処理あり）</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>11/3</t>
+          <t>9/20</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>文化の日</t>
+          <t>敬老の日</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>文化祭(音楽発表会)準備</t>
+          <t>ノー部活ウィーク</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>11/4に移動（要調整）</t>
+          <t>9/21に移動（要調整）</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>11/23</t>
+          <t>9/23</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>勤労感謝の日</t>
+          <t>秋分の日</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>学10</t>
+          <t>職8</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>11/24に移動（会議は木曜へ移す処理あり）</t>
+          <t>9/24に移動（会議は木曜へ移す処理あり）</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>1/10</t>
+          <t>11/3</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>成人の日</t>
+          <t>文化の日</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>ノー部活デー</t>
+          <t>文化祭(音楽発表会)準備</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>1/11に移動（要調整）</t>
+          <t>11/4に移動（要調整）</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2/11</t>
+          <t>11/23</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>建国記念の日</t>
+          <t>勤労感謝の日</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>↓【定時制１次入試】</t>
+          <t>学10</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>2/14に移動（要調整）</t>
+          <t>11/24に移動（会議は木曜へ移す処理あり）</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2/23</t>
+          <t>1/10</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>天皇誕生日</t>
+          <t>成人の日</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>【公立一般学力検査】</t>
+          <t>ノー部活デー</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>2/24に移動（要調整）</t>
+          <t>1/11に移動（要調整）</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>4/27</t>
+          <t>2/11</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>予</t>
+          <t>建国記念の日</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>会議</t>
+          <t>↓【定時制１次入試】</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>同じ週の木曜が休みのため移動できず（要調整）</t>
+          <t>2/14に移動（要調整）</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>4/30</t>
+          <t>2/23</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>運4</t>
+          <t>天皇誕生日</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>会議</t>
+          <t>【公立一般学力検査】</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>同じ週の木曜が休みのため移動できず（要調整）</t>
+          <t>2/24に移動（要調整）</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>9/24</t>
+          <t>4/27</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>職8</t>
+          <t>予</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -45678,12 +45658,12 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>1/7</t>
+          <t>4/30</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>卒認</t>
+          <t>運4</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -45700,20 +45680,42 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
+          <t>9/24</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>職8</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>会議</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>同じ週の木曜が休みのため移動できず（要調整）</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
           <t>1/7</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>職10</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr">
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>卒認</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
         <is>
           <t>会議</t>
         </is>
       </c>
-      <c r="D26" t="inlineStr">
+      <c r="D27" t="inlineStr">
         <is>
           <t>同じ週の木曜が休みのため移動できず（要調整）</t>
         </is>
@@ -45722,51 +45724,29 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>木曜に移した会議：35件</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>4/5(月)</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>部会</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>→</t>
-        </is>
-      </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>4/8(木)</t>
+          <t>1/7</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>職10</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>会議</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>同じ週の木曜が休みのため移動できず（要調整）</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>4/6(火)</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>努･採</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>→</t>
-        </is>
-      </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>4/8(木)</t>
+          <t>木曜に移した会議：34件</t>
         </is>
       </c>
     </row>
@@ -45778,7 +45758,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>運2</t>
+          <t>部会</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -45800,7 +45780,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>学3</t>
+          <t>努･採</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -45822,7 +45802,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>教</t>
+          <t>運2</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -45844,7 +45824,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>部会</t>
+          <t>職2</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -45866,7 +45846,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>運3</t>
+          <t>部会</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -45883,12 +45863,12 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>4/14(水)</t>
+          <t>4/12(月)</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>不</t>
+          <t>運3</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -45905,12 +45885,12 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>4/16(金)</t>
+          <t>4/14(水)</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>進1</t>
+          <t>不</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -45927,12 +45907,12 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>4/21(水)</t>
+          <t>4/16(金)</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>学4</t>
+          <t>進1</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -45942,19 +45922,19 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>4/22(木)</t>
+          <t>4/15(木)</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>5/10(月)</t>
+          <t>4/21(水)</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>職4</t>
+          <t>学4</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -45964,19 +45944,19 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>5/13(木)</t>
+          <t>4/22(木)</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>5/17(月)</t>
+          <t>5/10(月)</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>現2</t>
+          <t>職4</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -45986,19 +45966,19 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>5/20(木)</t>
+          <t>5/13(木)</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>5/24(月)</t>
+          <t>5/17(月)</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>職5</t>
+          <t>現2</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -46008,19 +45988,19 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>5/27(木)</t>
+          <t>5/20(木)</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>5/26(水)</t>
+          <t>5/24(月)</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>教科等研究部会</t>
+          <t>職5</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -46037,12 +46017,12 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>6/14(月)</t>
+          <t>5/26(水)</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>現3</t>
+          <t>教科等研究部会</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -46052,19 +46032,19 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>6/17(木)</t>
+          <t>5/27(木)</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>6/15(火)</t>
+          <t>6/14(月)</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>運6</t>
+          <t>現3</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -46081,12 +46061,12 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>6/28(月)</t>
+          <t>6/15(火)</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>職6</t>
+          <t>運6</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -46096,19 +46076,19 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>7/1(木)</t>
+          <t>6/17(木)</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>9/1(水)</t>
+          <t>6/28(月)</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>運7</t>
+          <t>職6</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -46118,7 +46098,7 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>9/2(木)</t>
+          <t>7/1(木)</t>
         </is>
       </c>
     </row>
@@ -46130,7 +46110,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>現4</t>
+          <t>運7</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -46147,12 +46127,12 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>9/6(月)</t>
+          <t>9/1(水)</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>学8</t>
+          <t>現4</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -46162,19 +46142,19 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>9/9(木)</t>
+          <t>9/2(木)</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>9/17(金)</t>
+          <t>9/6(月)</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>教</t>
+          <t>学8</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -46184,19 +46164,19 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>9/16(木)</t>
+          <t>9/9(木)</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>9/27(月)</t>
+          <t>9/17(金)</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>現5</t>
+          <t>教</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -46206,19 +46186,19 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>9/30(木)</t>
+          <t>9/16(木)</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>10/27(水)</t>
+          <t>9/27(月)</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>教支</t>
+          <t>現5</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -46228,19 +46208,19 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>10/28(木)</t>
+          <t>9/30(木)</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>11/5(金)</t>
+          <t>10/27(水)</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>運9</t>
+          <t>教支</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -46250,19 +46230,19 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>11/4(木)</t>
+          <t>10/28(木)</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>11/24(水)</t>
+          <t>11/5(金)</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>学10</t>
+          <t>運9</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -46272,19 +46252,19 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>11/25(木)</t>
+          <t>11/4(木)</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>12/10(金)</t>
+          <t>11/24(水)</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>進4</t>
+          <t>学10</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -46294,19 +46274,19 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>12/9(木)</t>
+          <t>11/25(木)</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>1/18(火)</t>
+          <t>12/10(金)</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>進5</t>
+          <t>進4</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -46316,19 +46296,19 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>1/20(木)</t>
+          <t>12/9(木)</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>1/31(月)</t>
+          <t>1/18(火)</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>部反②</t>
+          <t>進5</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -46338,19 +46318,19 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>2/3(木)</t>
+          <t>1/20(木)</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2/8(火)</t>
+          <t>1/31(月)</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>全反</t>
+          <t>部反②</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -46360,19 +46340,19 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>2/10(木)</t>
+          <t>2/3(木)</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>2/18(金)</t>
+          <t>2/8(火)</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>学12</t>
+          <t>全反</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
@@ -46382,19 +46362,19 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>2/17(木)</t>
+          <t>2/10(木)</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2/21(月)</t>
+          <t>2/18(金)</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>教</t>
+          <t>学12</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
@@ -46404,19 +46384,19 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>2/24(木)</t>
+          <t>2/17(木)</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>3/6(月)</t>
+          <t>2/21(月)</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>進認</t>
+          <t>教</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
@@ -46426,7 +46406,7 @@
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>3/9(木)</t>
+          <t>2/24(木)</t>
         </is>
       </c>
     </row>
@@ -46438,7 +46418,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>職11</t>
+          <t>進認</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -46455,12 +46435,12 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>3/10(金)</t>
+          <t>3/6(月)</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>編1</t>
+          <t>職11</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
@@ -46477,20 +46457,42 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
+          <t>3/10(金)</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>編1</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>→</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>3/9(木)</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
           <t>3/17(金)</t>
         </is>
       </c>
-      <c r="B63" t="inlineStr">
+      <c r="B64" t="inlineStr">
         <is>
           <t>採</t>
         </is>
       </c>
-      <c r="C63" t="inlineStr">
+      <c r="C64" t="inlineStr">
         <is>
           <t>→</t>
         </is>
       </c>
-      <c r="D63" t="inlineStr">
+      <c r="D64" t="inlineStr">
         <is>
           <t>3/16(木)</t>
         </is>

</xml_diff>

<commit_message>
Fix workbook view settings in FY2027 annual plan and add PDF
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FawjLRytv2ATkyFXeWDDqM
</commit_message>
<xml_diff>
--- a/令和9年度_年間計画（案）.xlsx
+++ b/令和9年度_年間計画（案）.xlsx
@@ -3,18 +3,13 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr codeName="ThisWorkbook"/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="2205" yWindow="2205" windowWidth="21600" windowHeight="11423" tabRatio="600" firstSheet="8" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="2205" yWindow="2205" windowWidth="21600" windowHeight="11423" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="年計" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="作成メモ・要確認" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xleta.TODAY" hidden="1" xlm="1">#NAME?</definedName>
-    <definedName name="Print_Area20">#REF!</definedName>
-    <definedName name="Print_Area2026">#REF!</definedName>
-    <definedName name="印刷範囲">#REF!</definedName>
-    <definedName name="印刷範囲" localSheetId="0">年計!$A$1:$AJ$65</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'年計'!$A$1:$AL$68</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -37268,7 +37263,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr codeName="Sheet1">
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:GJ84"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.68359375" defaultRowHeight="14.25"/>
@@ -40112,14 +40107,8 @@
       </c>
       <c r="AL21" s="446" t="n"/>
       <c r="AM21" s="447" t="n"/>
-      <c r="AQ21" s="418">
-        <f>_xlfn.WEBSERVICE("http://api.excelapi.org/datetime/holiday-list?year=2027&amp;line="&amp;ROW())</f>
-        <v/>
-      </c>
-      <c r="AR21" s="418">
-        <f>_xlfn.WEBSERVICE("http://api.excelapi.org/datetime/holiday?date="&amp;A1)</f>
-        <v/>
-      </c>
+      <c r="AQ21" s="418" t="n"/>
+      <c r="AR21" s="418" t="n"/>
       <c r="BA21" s="417" t="n"/>
     </row>
     <row r="22" ht="28.5" customFormat="1" customHeight="1" s="418">
@@ -45289,7 +45278,7 @@
   </mergeCells>
   <printOptions verticalCentered="1"/>
   <pageMargins left="0.4724409448818898" right="0.1968503937007874" top="0.3149606299212598" bottom="0.1968503937007874" header="0.2755905511811024" footer="0"/>
-  <pageSetup orientation="portrait" paperSize="9" scale="47"/>
+  <pageSetup orientation="landscape" paperSize="8" scale="47" fitToHeight="1" fitToWidth="1"/>
   <colBreaks count="1" manualBreakCount="1">
     <brk id="19" min="0" max="1048575" man="1"/>
   </colBreaks>

</xml_diff>

<commit_message>
Move school trip to 6/8-6/10 and reschedule related events
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FawjLRytv2ATkyFXeWDDqM
</commit_message>
<xml_diff>
--- a/令和9年度_年間計画（案）.xlsx
+++ b/令和9年度_年間計画（案）.xlsx
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="33">
+  <fonts count="36">
     <font>
       <name val="ＭＳ 明朝"/>
       <charset val="128"/>
@@ -246,6 +246,20 @@
       <charset val="128"/>
       <family val="3"/>
       <color rgb="FFFFC000"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="ＭＳ Ｐゴシック"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="ＭＳ Ｐゴシック"/>
+      <color rgb="FFFFC000"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="ＭＳ Ｐゴシック"/>
+      <color rgb="FFFF0000"/>
       <sz val="12"/>
     </font>
   </fonts>
@@ -1175,7 +1189,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="31" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="413">
+  <cellXfs count="423">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <protection locked="0" hidden="0"/>
     </xf>
@@ -2362,6 +2376,36 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="75" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="2">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="33" fillId="0" borderId="26" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="2">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="33" fillId="0" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="2">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="33" fillId="0" borderId="32" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="2">
+      <alignment vertical="center" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="33" fillId="0" borderId="26" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="2">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="33" fillId="0" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="2">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="33" fillId="0" borderId="32" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="2">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="33" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="2">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="34" fillId="0" borderId="26" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="2">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="33" fillId="0" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="2">
+      <alignment vertical="center" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="35" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="2">
+      <alignment vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="4">
@@ -4816,7 +4860,11 @@
       <c r="H16" s="65" t="n">
         <v>7</v>
       </c>
-      <c r="I16" s="16" t="n"/>
+      <c r="I16" s="413" t="inlineStr">
+        <is>
+          <t>修学旅行事前指導(3年)</t>
+        </is>
+      </c>
       <c r="J16" s="147" t="inlineStr">
         <is>
           <t>委</t>
@@ -5134,9 +5182,9 @@
       <c r="H18" s="65" t="n">
         <v>8</v>
       </c>
-      <c r="I18" s="206" t="inlineStr">
-        <is>
-          <t>耳鼻科検診(1年午後)</t>
+      <c r="I18" s="413" t="inlineStr">
+        <is>
+          <t>修学旅行(３年)</t>
         </is>
       </c>
       <c r="J18" s="76" t="n"/>
@@ -5264,7 +5312,11 @@
           <t>火</t>
         </is>
       </c>
-      <c r="I19" s="18" t="n"/>
+      <c r="I19" s="414" t="inlineStr">
+        <is>
+          <t>｜</t>
+        </is>
+      </c>
       <c r="J19" s="38" t="n"/>
       <c r="K19" s="57" t="inlineStr">
         <is>
@@ -5358,9 +5410,9 @@
       <c r="H20" s="52" t="n">
         <v>9</v>
       </c>
-      <c r="I20" s="280" t="inlineStr">
-        <is>
-          <t>耳鼻科検診</t>
+      <c r="I20" s="415" t="inlineStr">
+        <is>
+          <t>｜</t>
         </is>
       </c>
       <c r="J20" s="53" t="n"/>
@@ -5476,9 +5528,9 @@
           <t>水</t>
         </is>
       </c>
-      <c r="I21" s="211" t="inlineStr">
-        <is>
-          <t>(IJ･2･3年抽出午後)</t>
+      <c r="I21" s="414" t="inlineStr">
+        <is>
+          <t>｜</t>
         </is>
       </c>
       <c r="J21" s="38" t="n"/>
@@ -5597,9 +5649,9 @@
       <c r="H22" s="52" t="n">
         <v>10</v>
       </c>
-      <c r="I22" s="234" t="inlineStr">
-        <is>
-          <t>歯科健診(1年午前)</t>
+      <c r="I22" s="416" t="inlineStr">
+        <is>
+          <t>↓</t>
         </is>
       </c>
       <c r="J22" s="140" t="n"/>
@@ -5693,7 +5745,7 @@
           <t>木</t>
         </is>
       </c>
-      <c r="I23" s="138" t="n"/>
+      <c r="I23" s="417" t="n"/>
       <c r="J23" s="38" t="n"/>
       <c r="K23" s="203" t="inlineStr">
         <is>
@@ -5781,11 +5833,7 @@
       <c r="H24" s="52" t="n">
         <v>11</v>
       </c>
-      <c r="I24" s="206" t="inlineStr">
-        <is>
-          <t>修学旅行事前指導(3年)</t>
-        </is>
-      </c>
+      <c r="I24" s="413" t="n"/>
       <c r="J24" s="53" t="inlineStr">
         <is>
           <t>定</t>
@@ -6412,11 +6460,7 @@
       <c r="H30" s="65" t="n">
         <v>14</v>
       </c>
-      <c r="I30" s="206" t="inlineStr">
-        <is>
-          <t>修学旅行(３年)</t>
-        </is>
-      </c>
+      <c r="I30" s="413" t="n"/>
       <c r="J30" s="147" t="n"/>
       <c r="K30" s="52" t="n">
         <v>14</v>
@@ -6524,9 +6568,9 @@
           <t>月</t>
         </is>
       </c>
-      <c r="I31" s="211" t="inlineStr">
-        <is>
-          <t>｜ノー部活デー</t>
+      <c r="I31" s="414" t="inlineStr">
+        <is>
+          <t>ノー部活デー</t>
         </is>
       </c>
       <c r="J31" s="72" t="n"/>
@@ -6631,9 +6675,9 @@
       <c r="H32" s="65" t="n">
         <v>15</v>
       </c>
-      <c r="I32" s="206" t="inlineStr">
-        <is>
-          <t>｜│</t>
+      <c r="I32" s="413" t="inlineStr">
+        <is>
+          <t>耳鼻科検診(1年午後)</t>
         </is>
       </c>
       <c r="J32" s="53" t="n"/>
@@ -6746,11 +6790,7 @@
           <t>火</t>
         </is>
       </c>
-      <c r="I33" s="211" t="inlineStr">
-        <is>
-          <t>｜│</t>
-        </is>
-      </c>
+      <c r="I33" s="414" t="n"/>
       <c r="J33" s="38" t="n"/>
       <c r="K33" s="57" t="inlineStr">
         <is>
@@ -6846,9 +6886,9 @@
       <c r="H34" s="52" t="n">
         <v>16</v>
       </c>
-      <c r="I34" s="319" t="inlineStr">
-        <is>
-          <t>｜│</t>
+      <c r="I34" s="418" t="inlineStr">
+        <is>
+          <t>耳鼻科検診</t>
         </is>
       </c>
       <c r="J34" s="53" t="n"/>
@@ -6958,9 +6998,9 @@
           <t>水</t>
         </is>
       </c>
-      <c r="I35" s="320" t="inlineStr">
-        <is>
-          <t>↓↓</t>
+      <c r="I35" s="419" t="inlineStr">
+        <is>
+          <t>(IJ･2･3年抽出午後)</t>
         </is>
       </c>
       <c r="J35" s="61" t="n"/>
@@ -7069,7 +7109,11 @@
       <c r="H36" s="52" t="n">
         <v>17</v>
       </c>
-      <c r="I36" s="75" t="n"/>
+      <c r="I36" s="416" t="inlineStr">
+        <is>
+          <t>歯科健診(1年午前)</t>
+        </is>
+      </c>
       <c r="J36" s="38" t="inlineStr">
         <is>
           <t>学6(2年)
@@ -7876,11 +7920,7 @@
       <c r="B44" s="65" t="n">
         <v>21</v>
       </c>
-      <c r="C44" s="389" t="inlineStr">
-        <is>
-          <t>稲武野外学習説明会(2年)</t>
-        </is>
-      </c>
+      <c r="C44" s="414" t="n"/>
       <c r="D44" s="53" t="n"/>
       <c r="E44" s="52" t="n">
         <v>21</v>
@@ -8082,7 +8122,11 @@
       <c r="H46" s="65" t="n">
         <v>22</v>
       </c>
-      <c r="I46" s="16" t="n"/>
+      <c r="I46" s="420" t="inlineStr">
+        <is>
+          <t>稲武野外学習説明会(2年)</t>
+        </is>
+      </c>
       <c r="J46" s="53" t="n"/>
       <c r="K46" s="52" t="n">
         <v>22</v>
@@ -8655,11 +8699,7 @@
       <c r="E52" s="65" t="n">
         <v>25</v>
       </c>
-      <c r="F52" s="206" t="inlineStr">
-        <is>
-          <t>稲武事前指導(2年)</t>
-        </is>
-      </c>
+      <c r="F52" s="413" t="n"/>
       <c r="G52" s="53" t="n"/>
       <c r="H52" s="97" t="n">
         <v>25</v>
@@ -8866,11 +8906,7 @@
       <c r="E54" s="52" t="n">
         <v>26</v>
       </c>
-      <c r="F54" s="280" t="inlineStr">
-        <is>
-          <t>稲武野外学習(2年)</t>
-        </is>
-      </c>
+      <c r="F54" s="415" t="n"/>
       <c r="G54" s="91" t="n"/>
       <c r="H54" s="221" t="n">
         <v>26</v>
@@ -9068,11 +9104,7 @@
       <c r="E56" s="52" t="n">
         <v>27</v>
       </c>
-      <c r="F56" s="352" t="inlineStr">
-        <is>
-          <t>稲武野外学習(2年)</t>
-        </is>
-      </c>
+      <c r="F56" s="421" t="n"/>
       <c r="G56" s="87" t="inlineStr">
         <is>
           <t>職5</t>
@@ -9270,11 +9302,7 @@
       <c r="E58" s="52" t="n">
         <v>28</v>
       </c>
-      <c r="F58" s="352" t="inlineStr">
-        <is>
-          <t>稲武野外学習(2年)</t>
-        </is>
-      </c>
+      <c r="F58" s="421" t="n"/>
       <c r="G58" s="82" t="inlineStr">
         <is>
           <t>第１回NCS会議</t>
@@ -10226,7 +10254,11 @@
       <c r="H68" s="27" t="n"/>
       <c r="I68" s="26" t="n"/>
       <c r="J68" s="26" t="n"/>
-      <c r="K68" s="27" t="n"/>
+      <c r="K68" s="422" t="inlineStr">
+        <is>
+          <t>稲武野外学習(2年)：7〜8月に実施予定（日程未定）</t>
+        </is>
+      </c>
       <c r="L68" s="27" t="n"/>
       <c r="M68" s="27" t="n"/>
       <c r="N68" s="27" t="n"/>
@@ -10780,7 +10812,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D64"/>
+  <dimension ref="A1:D70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16.15"/>
   <cols>
     <col width="14" customWidth="1" style="201" min="1" max="1"/>
@@ -10859,7 +10891,6 @@
         </is>
       </c>
     </row>
-    <row r="11"/>
     <row r="12">
       <c r="A12" s="0" t="inlineStr">
         <is>
@@ -11222,7 +11253,6 @@
         </is>
       </c>
     </row>
-    <row r="29"/>
     <row r="30">
       <c r="A30" s="0" t="inlineStr">
         <is>
@@ -11975,6 +12005,41 @@
       <c r="D64" s="0" t="inlineStr">
         <is>
           <t>3/16(木)</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>学校の指示で修正した点</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>・修学旅行(3年)を6/8(火)〜6/10(木)に変更。その週の健診（耳鼻科・歯科）は6/15〜6/17の同じ曜日へ移動。</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>・修学旅行事前指導(3年)は出発前の6/7(月)へ移動（要確認）。心臓検診(1年)は6/11(金)のまま。</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>・稲武野外学習(2年)と事前指導を5月から削除。7〜8月実施予定（日程未定）。</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>・稲武野外学習説明会(2年)を6/22(火)へ移動（6月下旬で調整中）。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Replace span arrows with repeated entries; move trip briefing to 5/6; drop Rikuzentakata exchange
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FawjLRytv2ATkyFXeWDDqM
</commit_message>
<xml_diff>
--- a/令和9年度_年間計画（案）.xlsx
+++ b/令和9年度_年間計画（案）.xlsx
@@ -1189,7 +1189,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="31" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="423">
+  <cellXfs count="424">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <protection locked="0" hidden="0"/>
     </xf>
@@ -2406,6 +2406,9 @@
     </xf>
     <xf numFmtId="1" fontId="35" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="2">
       <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="1" fontId="33" fillId="0" borderId="26" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="2">
+      <alignment horizontal="justify" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="4">
@@ -3092,7 +3095,7 @@
       </c>
       <c r="I4" s="206" t="inlineStr">
         <is>
-          <t>｜</t>
+          <t>教育相談（全学年）</t>
         </is>
       </c>
       <c r="J4" s="104" t="n"/>
@@ -3208,7 +3211,7 @@
       </c>
       <c r="I5" s="211" t="inlineStr">
         <is>
-          <t>｜</t>
+          <t>ノー部活ウィーク</t>
         </is>
       </c>
       <c r="J5" s="79" t="n"/>
@@ -3262,7 +3265,7 @@
       </c>
       <c r="AA5" s="211" t="inlineStr">
         <is>
-          <t>｜　　1･2年成績一覧表提出</t>
+          <t>1･2年成績一覧表提出</t>
         </is>
       </c>
       <c r="AB5" s="61" t="n"/>
@@ -3278,11 +3281,7 @@
           <t>火</t>
         </is>
       </c>
-      <c r="AG5" s="220" t="inlineStr">
-        <is>
-          <t>│</t>
-        </is>
-      </c>
+      <c r="AG5" s="220" t="n"/>
       <c r="AH5" s="131" t="n"/>
       <c r="AI5" s="57" t="inlineStr">
         <is>
@@ -3363,7 +3362,7 @@
       </c>
       <c r="I6" s="206" t="inlineStr">
         <is>
-          <t>｜</t>
+          <t>教育相談（全学年）</t>
         </is>
       </c>
       <c r="J6" s="166" t="n"/>
@@ -3406,25 +3405,21 @@
       </c>
       <c r="AA6" s="206" t="inlineStr">
         <is>
-          <t>｜</t>
+          <t>保護者会(全)</t>
         </is>
       </c>
       <c r="AB6" s="133" t="n"/>
       <c r="AC6" s="221" t="n">
         <v>2</v>
       </c>
-      <c r="AD6" s="226" t="inlineStr">
-        <is>
-          <t>｜</t>
-        </is>
-      </c>
+      <c r="AD6" s="226" t="n"/>
       <c r="AE6" s="209" t="n"/>
       <c r="AF6" s="52" t="n">
         <v>2</v>
       </c>
       <c r="AG6" s="227" t="inlineStr">
         <is>
-          <t>│</t>
+          <t>ノー部活ウィーク</t>
         </is>
       </c>
       <c r="AH6" s="132" t="n"/>
@@ -3518,7 +3513,7 @@
       </c>
       <c r="I7" s="211" t="inlineStr">
         <is>
-          <t>｜</t>
+          <t>ノー部活ウィーク</t>
         </is>
       </c>
       <c r="J7" s="96" t="n"/>
@@ -3568,7 +3563,7 @@
       </c>
       <c r="AA7" s="231" t="inlineStr">
         <is>
-          <t>｜　  第２回いじめ防対会議</t>
+          <t>第２回いじめ防対会議</t>
         </is>
       </c>
       <c r="AC7" s="203" t="inlineStr">
@@ -3576,11 +3571,7 @@
           <t>日</t>
         </is>
       </c>
-      <c r="AD7" s="232" t="inlineStr">
-        <is>
-          <t>↓</t>
-        </is>
-      </c>
+      <c r="AD7" s="232" t="n"/>
       <c r="AE7" s="218" t="n"/>
       <c r="AF7" s="57" t="inlineStr">
         <is>
@@ -3589,7 +3580,7 @@
       </c>
       <c r="AG7" s="211" t="inlineStr">
         <is>
-          <t>│　　 　　　第２回NCS会議</t>
+          <t>第２回NCS会議</t>
         </is>
       </c>
       <c r="AH7" s="159" t="n"/>
@@ -3679,7 +3670,7 @@
       </c>
       <c r="I8" s="234" t="inlineStr">
         <is>
-          <t>｜歯科健診(IJ･2年午前)</t>
+          <t>教育相談（全学年）</t>
         </is>
       </c>
       <c r="J8" s="104" t="n"/>
@@ -3725,7 +3716,7 @@
       </c>
       <c r="AA8" s="206" t="inlineStr">
         <is>
-          <t>｜</t>
+          <t>保護者会(全)</t>
         </is>
       </c>
       <c r="AB8" s="53" t="n"/>
@@ -3739,7 +3730,7 @@
       </c>
       <c r="AG8" s="206" t="inlineStr">
         <is>
-          <t>│</t>
+          <t>ノー部活ウィーク</t>
         </is>
       </c>
       <c r="AH8" s="76" t="inlineStr">
@@ -3841,7 +3832,7 @@
       </c>
       <c r="I9" s="219" t="inlineStr">
         <is>
-          <t>｜                　学6(1･3年)</t>
+          <t>ノー部活ウィーク・歯科健診(IJ･2年午前)・学6(1･3年)</t>
         </is>
       </c>
       <c r="J9" s="157" t="n"/>
@@ -3885,11 +3876,7 @@
           <t>金</t>
         </is>
       </c>
-      <c r="AA9" s="211" t="inlineStr">
-        <is>
-          <t>｜</t>
-        </is>
-      </c>
+      <c r="AA9" s="211" t="n"/>
       <c r="AB9" s="69" t="n"/>
       <c r="AC9" s="57" t="inlineStr">
         <is>
@@ -3905,7 +3892,7 @@
       </c>
       <c r="AG9" s="211" t="inlineStr">
         <is>
-          <t>│【公立推薦･特色入試】</t>
+          <t>【公立推薦･特色入試】</t>
         </is>
       </c>
       <c r="AH9" s="38" t="n"/>
@@ -3999,7 +3986,7 @@
       </c>
       <c r="I10" s="242" t="inlineStr">
         <is>
-          <t>｜</t>
+          <t>教育相談（全学年）</t>
         </is>
       </c>
       <c r="K10" s="207" t="n">
@@ -4050,7 +4037,7 @@
       </c>
       <c r="AG10" s="206" t="inlineStr">
         <is>
-          <t>│</t>
+          <t>ノー部活ウィーク</t>
         </is>
       </c>
       <c r="AH10" s="76" t="n"/>
@@ -4140,7 +4127,7 @@
       </c>
       <c r="I11" s="211" t="inlineStr">
         <is>
-          <t>↓</t>
+          <t>ノー部活ウィーク</t>
         </is>
       </c>
       <c r="J11" s="58" t="n"/>
@@ -4202,11 +4189,7 @@
           <t>金</t>
         </is>
       </c>
-      <c r="AG11" s="220" t="inlineStr">
-        <is>
-          <t>│</t>
-        </is>
-      </c>
+      <c r="AG11" s="220" t="n"/>
       <c r="AH11" s="61" t="n"/>
       <c r="AI11" s="203" t="inlineStr">
         <is>
@@ -4344,11 +4327,7 @@
       <c r="AF12" s="221" t="n">
         <v>5</v>
       </c>
-      <c r="AG12" s="255" t="inlineStr">
-        <is>
-          <t>│</t>
-        </is>
-      </c>
+      <c r="AG12" s="255" t="n"/>
       <c r="AH12" s="247" t="n"/>
       <c r="AI12" s="221" t="n">
         <v>5</v>
@@ -4431,7 +4410,7 @@
       </c>
       <c r="L13" s="211" t="inlineStr">
         <is>
-          <t>｜　　　　　成績一覧表提出</t>
+          <t>成績一覧表提出</t>
         </is>
       </c>
       <c r="M13" s="72" t="n"/>
@@ -4482,11 +4461,7 @@
           <t>土</t>
         </is>
       </c>
-      <c r="AG13" s="259" t="inlineStr">
-        <is>
-          <t>│</t>
-        </is>
-      </c>
+      <c r="AG13" s="259" t="n"/>
       <c r="AH13" s="230" t="n"/>
       <c r="AI13" s="203" t="inlineStr">
         <is>
@@ -4575,7 +4550,7 @@
       </c>
       <c r="L14" s="206" t="inlineStr">
         <is>
-          <t>｜</t>
+          <t>保護者会（全）</t>
         </is>
       </c>
       <c r="M14" s="53" t="n"/>
@@ -4612,7 +4587,7 @@
       </c>
       <c r="AA14" s="206" t="inlineStr">
         <is>
-          <t>｜</t>
+          <t>保護者会(全)</t>
         </is>
       </c>
       <c r="AB14" s="147" t="n"/>
@@ -4624,11 +4599,7 @@
       <c r="AF14" s="221" t="n">
         <v>6</v>
       </c>
-      <c r="AG14" s="255" t="inlineStr">
-        <is>
-          <t>│</t>
-        </is>
-      </c>
+      <c r="AG14" s="255" t="n"/>
       <c r="AH14" s="249" t="n"/>
       <c r="AI14" s="52" t="n">
         <v>6</v>
@@ -4701,7 +4672,7 @@
       </c>
       <c r="F15" s="264" t="inlineStr">
         <is>
-          <t>新体力テスト準備</t>
+          <t>新体力テスト準備・⑤⑥修学旅行・進路説明会(3年)</t>
         </is>
       </c>
       <c r="G15" s="61" t="n"/>
@@ -4719,7 +4690,7 @@
       </c>
       <c r="L15" s="211" t="inlineStr">
         <is>
-          <t>｜　 第１回いじめ防対会議</t>
+          <t>第１回いじめ防対会議</t>
         </is>
       </c>
       <c r="M15" s="38" t="n"/>
@@ -4756,11 +4727,7 @@
           <t>月</t>
         </is>
       </c>
-      <c r="AA15" s="211" t="inlineStr">
-        <is>
-          <t>｜</t>
-        </is>
-      </c>
+      <c r="AA15" s="211" t="n"/>
       <c r="AB15" s="72" t="n"/>
       <c r="AC15" s="57" t="inlineStr">
         <is>
@@ -4774,11 +4741,7 @@
           <t>日</t>
         </is>
       </c>
-      <c r="AG15" s="265" t="inlineStr">
-        <is>
-          <t>│</t>
-        </is>
-      </c>
+      <c r="AG15" s="265" t="n"/>
       <c r="AH15" s="230" t="n"/>
       <c r="AI15" s="57" t="inlineStr">
         <is>
@@ -4875,7 +4838,7 @@
       </c>
       <c r="L16" s="206" t="inlineStr">
         <is>
-          <t>｜</t>
+          <t>保護者会（全）</t>
         </is>
       </c>
       <c r="M16" s="53" t="n"/>
@@ -4916,7 +4879,7 @@
       </c>
       <c r="AA16" s="227" t="inlineStr">
         <is>
-          <t>｜</t>
+          <t>保護者会(全)</t>
         </is>
       </c>
       <c r="AB16" s="53" t="n"/>
@@ -4938,7 +4901,7 @@
       </c>
       <c r="AG16" s="206" t="inlineStr">
         <is>
-          <t>│</t>
+          <t>ノー部活ウィーク</t>
         </is>
       </c>
       <c r="AH16" s="132" t="inlineStr">
@@ -5032,7 +4995,7 @@
       </c>
       <c r="L17" s="267" t="inlineStr">
         <is>
-          <t>｜　　　　　通知表（仮）提出</t>
+          <t>通知表（仮）提出</t>
         </is>
       </c>
       <c r="N17" s="203" t="inlineStr">
@@ -5078,7 +5041,7 @@
       </c>
       <c r="AA17" s="211" t="inlineStr">
         <is>
-          <t>↓　　　　　　通知表(仮)提出</t>
+          <t>通知表(仮)提出</t>
         </is>
       </c>
       <c r="AB17" s="38" t="n"/>
@@ -5104,7 +5067,7 @@
       </c>
       <c r="AG17" s="219" t="inlineStr">
         <is>
-          <t>↓【公立推薦･特色合格発表】</t>
+          <t>【公立推薦･特色合格発表】</t>
         </is>
       </c>
       <c r="AH17" s="61" t="n"/>
@@ -5193,7 +5156,7 @@
       </c>
       <c r="L18" s="234" t="inlineStr">
         <is>
-          <t>｜</t>
+          <t>保護者会（全）</t>
         </is>
       </c>
       <c r="M18" s="53" t="n"/>
@@ -5312,22 +5275,14 @@
           <t>火</t>
         </is>
       </c>
-      <c r="I19" s="414" t="inlineStr">
-        <is>
-          <t>｜</t>
-        </is>
-      </c>
+      <c r="I19" s="414" t="n"/>
       <c r="J19" s="38" t="n"/>
       <c r="K19" s="57" t="inlineStr">
         <is>
           <t>木</t>
         </is>
       </c>
-      <c r="L19" s="231" t="inlineStr">
-        <is>
-          <t>｜</t>
-        </is>
-      </c>
+      <c r="L19" s="231" t="n"/>
       <c r="N19" s="203" t="inlineStr">
         <is>
           <t>日</t>
@@ -5377,7 +5332,7 @@
       </c>
       <c r="AG19" s="279" t="inlineStr">
         <is>
-          <t>│ノー部活デー</t>
+          <t>ノー部活デー</t>
         </is>
       </c>
       <c r="AI19" s="57" t="inlineStr">
@@ -5412,7 +5367,7 @@
       </c>
       <c r="I20" s="415" t="inlineStr">
         <is>
-          <t>｜</t>
+          <t>修学旅行(３年)</t>
         </is>
       </c>
       <c r="J20" s="53" t="n"/>
@@ -5421,7 +5376,7 @@
       </c>
       <c r="L20" s="211" t="inlineStr">
         <is>
-          <t>｜</t>
+          <t>保護者会（全）</t>
         </is>
       </c>
       <c r="M20" s="53" t="n"/>
@@ -5453,9 +5408,7 @@
       </c>
       <c r="X20" s="283" t="inlineStr">
         <is>
-          <t>保護者会(3年)
-教育相談(1・2年)
-│ノー部活ウィーク</t>
+          <t>保護者会(3年)</t>
         </is>
       </c>
       <c r="Y20" s="53" t="n"/>
@@ -5478,7 +5431,7 @@
       </c>
       <c r="AG20" s="276" t="inlineStr">
         <is>
-          <t>│ノー部活デー</t>
+          <t>学年末テスト(１･２年)</t>
         </is>
       </c>
       <c r="AH20" s="141" t="n"/>
@@ -5528,22 +5481,14 @@
           <t>水</t>
         </is>
       </c>
-      <c r="I21" s="414" t="inlineStr">
-        <is>
-          <t>｜</t>
-        </is>
-      </c>
+      <c r="I21" s="414" t="n"/>
       <c r="J21" s="38" t="n"/>
       <c r="K21" s="57" t="inlineStr">
         <is>
           <t>金</t>
         </is>
       </c>
-      <c r="L21" s="211" t="inlineStr">
-        <is>
-          <t xml:space="preserve">↓　　　　</t>
-        </is>
-      </c>
+      <c r="L21" s="211" t="n"/>
       <c r="M21" s="38" t="n"/>
       <c r="N21" s="57" t="inlineStr">
         <is>
@@ -5579,7 +5524,11 @@
           <t>火</t>
         </is>
       </c>
-      <c r="X21" s="136" t="n"/>
+      <c r="X21" s="136" t="inlineStr">
+        <is>
+          <t>教育相談(1・2年)・ノー部活ウィーク</t>
+        </is>
+      </c>
       <c r="Y21" s="85" t="n"/>
       <c r="Z21" s="57" t="inlineStr">
         <is>
@@ -5606,7 +5555,7 @@
       </c>
       <c r="AG21" s="211" t="inlineStr">
         <is>
-          <t>│</t>
+          <t>ノー部活デー</t>
         </is>
       </c>
       <c r="AH21" s="38" t="n"/>
@@ -5651,7 +5600,7 @@
       </c>
       <c r="I22" s="416" t="inlineStr">
         <is>
-          <t>↓</t>
+          <t>修学旅行(３年)</t>
         </is>
       </c>
       <c r="J22" s="140" t="n"/>
@@ -5665,7 +5614,7 @@
       </c>
       <c r="O22" s="227" t="inlineStr">
         <is>
-          <t>│</t>
+          <t>学校閉庁日</t>
         </is>
       </c>
       <c r="P22" s="81" t="n"/>
@@ -5684,7 +5633,7 @@
       </c>
       <c r="X22" s="290" t="inlineStr">
         <is>
-          <t>││</t>
+          <t>保護者会(3年)</t>
         </is>
       </c>
       <c r="Y22" s="38" t="n"/>
@@ -5707,7 +5656,7 @@
       </c>
       <c r="AG22" s="206" t="inlineStr">
         <is>
-          <t>│</t>
+          <t>学年末テスト(１･２年)</t>
         </is>
       </c>
       <c r="AH22" s="76" t="inlineStr">
@@ -5759,7 +5708,11 @@
           <t>火</t>
         </is>
       </c>
-      <c r="O23" s="68" t="n"/>
+      <c r="O23" s="68" t="inlineStr">
+        <is>
+          <t>ノー部活ウィーク</t>
+        </is>
+      </c>
       <c r="P23" s="78" t="n"/>
       <c r="Q23" s="62" t="inlineStr">
         <is>
@@ -5782,7 +5735,7 @@
       </c>
       <c r="X23" s="294" t="inlineStr">
         <is>
-          <t>││</t>
+          <t>教育相談(1・2年)・ノー部活ウィーク</t>
         </is>
       </c>
       <c r="Y23" s="61" t="n"/>
@@ -5872,7 +5825,7 @@
       </c>
       <c r="X24" s="299" t="inlineStr">
         <is>
-          <t>││</t>
+          <t>保護者会(3年)</t>
         </is>
       </c>
       <c r="Y24" s="72" t="n"/>
@@ -5890,7 +5843,7 @@
       </c>
       <c r="AD24" s="300" t="inlineStr">
         <is>
-          <t>※ノー部活デー</t>
+          <t>保護者会(3年)</t>
         </is>
       </c>
       <c r="AE24" s="145" t="n"/>
@@ -5974,7 +5927,7 @@
       </c>
       <c r="X25" s="219" t="inlineStr">
         <is>
-          <t>││</t>
+          <t>教育相談(1・2年)・ノー部活ウィーク</t>
         </is>
       </c>
       <c r="Y25" s="69" t="n"/>
@@ -5992,7 +5945,7 @@
       </c>
       <c r="AD25" s="211" t="inlineStr">
         <is>
-          <t>保護者会(3年)・│</t>
+          <t>ノー部活デー</t>
         </is>
       </c>
       <c r="AE25" s="132" t="n"/>
@@ -6061,7 +6014,7 @@
       </c>
       <c r="O26" s="227" t="inlineStr">
         <is>
-          <t>│</t>
+          <t>学校閉庁日</t>
         </is>
       </c>
       <c r="P26" s="81" t="n"/>
@@ -6080,7 +6033,7 @@
       </c>
       <c r="X26" s="299" t="inlineStr">
         <is>
-          <t>││</t>
+          <t>保護者会(3年)</t>
         </is>
       </c>
       <c r="Y26" s="133" t="inlineStr">
@@ -6098,7 +6051,7 @@
       </c>
       <c r="AD26" s="234" t="inlineStr">
         <is>
-          <t>｜</t>
+          <t>保護者会(3年)</t>
         </is>
       </c>
       <c r="AE26" s="76" t="n"/>
@@ -6161,7 +6114,7 @@
       </c>
       <c r="O27" s="211" t="inlineStr">
         <is>
-          <t>│</t>
+          <t>ノー部活ウィーク</t>
         </is>
       </c>
       <c r="P27" s="78" t="n"/>
@@ -6186,7 +6139,7 @@
       </c>
       <c r="X27" s="219" t="inlineStr">
         <is>
-          <t>↓↓</t>
+          <t>教育相談(1・2年)・ノー部活ウィーク</t>
         </is>
       </c>
       <c r="Y27" s="61" t="n"/>
@@ -6204,7 +6157,7 @@
       </c>
       <c r="AD27" s="211" t="inlineStr">
         <is>
-          <t>｜【私立専修推薦･特色入試】</t>
+          <t>【私立専修推薦･特色入試】</t>
         </is>
       </c>
       <c r="AE27" s="38" t="n"/>
@@ -6261,7 +6214,7 @@
       </c>
       <c r="O28" s="227" t="inlineStr">
         <is>
-          <t>│</t>
+          <t>学校閉庁日</t>
         </is>
       </c>
       <c r="P28" s="81" t="n"/>
@@ -6278,11 +6231,7 @@
       <c r="W28" s="221" t="n">
         <v>13</v>
       </c>
-      <c r="X28" s="232" t="inlineStr">
-        <is>
-          <t>││</t>
-        </is>
-      </c>
+      <c r="X28" s="232" t="n"/>
       <c r="Y28" s="218" t="n"/>
       <c r="Z28" s="65" t="n">
         <v>13</v>
@@ -6298,7 +6247,7 @@
       </c>
       <c r="AD28" s="234" t="inlineStr">
         <is>
-          <t>｜</t>
+          <t>保護者会(3年)</t>
         </is>
       </c>
       <c r="AE28" s="53" t="n"/>
@@ -6373,7 +6322,7 @@
       </c>
       <c r="O29" s="211" t="inlineStr">
         <is>
-          <t>↓</t>
+          <t>ノー部活ウィーク</t>
         </is>
       </c>
       <c r="P29" s="78" t="n"/>
@@ -6396,11 +6345,7 @@
           <t>土</t>
         </is>
       </c>
-      <c r="X29" s="265" t="inlineStr">
-        <is>
-          <t>││</t>
-        </is>
-      </c>
+      <c r="X29" s="265" t="n"/>
       <c r="Y29" s="218" t="n"/>
       <c r="Z29" s="62" t="inlineStr">
         <is>
@@ -6414,11 +6359,7 @@
           <t>木</t>
         </is>
       </c>
-      <c r="AD29" s="314" t="inlineStr">
-        <is>
-          <t>｜</t>
-        </is>
-      </c>
+      <c r="AD29" s="314" t="n"/>
       <c r="AF29" s="203" t="inlineStr">
         <is>
           <t>日</t>
@@ -6493,11 +6434,7 @@
       <c r="W30" s="207" t="n">
         <v>14</v>
       </c>
-      <c r="X30" s="255" t="inlineStr">
-        <is>
-          <t>││</t>
-        </is>
-      </c>
+      <c r="X30" s="255" t="n"/>
       <c r="Y30" s="209" t="n"/>
       <c r="Z30" s="52" t="n">
         <v>14</v>
@@ -6509,7 +6446,7 @@
       </c>
       <c r="AD30" s="206" t="inlineStr">
         <is>
-          <t xml:space="preserve">｜　　</t>
+          <t>保護者会(3年)</t>
         </is>
       </c>
       <c r="AE30" s="53" t="inlineStr">
@@ -6522,7 +6459,7 @@
       </c>
       <c r="AG30" s="307" t="inlineStr">
         <is>
-          <t>※↓【定時制１次入試】</t>
+          <t>※【定時制１次入試】</t>
         </is>
       </c>
       <c r="AH30" s="53" t="inlineStr">
@@ -6607,11 +6544,7 @@
           <t>日</t>
         </is>
       </c>
-      <c r="X31" s="232" t="inlineStr">
-        <is>
-          <t>││</t>
-        </is>
-      </c>
+      <c r="X31" s="232" t="n"/>
       <c r="Y31" s="218" t="n"/>
       <c r="Z31" s="57" t="inlineStr">
         <is>
@@ -6625,11 +6558,7 @@
           <t>金</t>
         </is>
       </c>
-      <c r="AD31" s="211" t="inlineStr">
-        <is>
-          <t xml:space="preserve">↓　　</t>
-        </is>
-      </c>
+      <c r="AD31" s="211" t="n"/>
       <c r="AE31" s="72" t="n"/>
       <c r="AF31" s="57" t="inlineStr">
         <is>
@@ -6718,7 +6647,7 @@
       </c>
       <c r="X32" s="206" t="inlineStr">
         <is>
-          <t>││</t>
+          <t>保護者会(3年)</t>
         </is>
       </c>
       <c r="Y32" s="147" t="n"/>
@@ -6831,7 +6760,7 @@
       </c>
       <c r="X33" s="211" t="inlineStr">
         <is>
-          <t>↓↓</t>
+          <t>教育相談(1・2年)・ノー部活ウィーク</t>
         </is>
       </c>
       <c r="Y33" s="72" t="n"/>
@@ -6900,11 +6829,7 @@
       <c r="N34" s="65" t="n">
         <v>16</v>
       </c>
-      <c r="O34" s="206" t="inlineStr">
-        <is>
-          <t>陸前高田市交流(2年)</t>
-        </is>
-      </c>
+      <c r="O34" s="206" t="n"/>
       <c r="P34" s="147" t="n"/>
       <c r="Q34" s="65" t="n">
         <v>16</v>
@@ -6929,7 +6854,7 @@
       </c>
       <c r="X34" s="211" t="inlineStr">
         <is>
-          <t xml:space="preserve">期末テスト </t>
+          <t>期末テスト</t>
         </is>
       </c>
       <c r="Y34" s="53" t="n"/>
@@ -7016,11 +6941,7 @@
           <t>月</t>
         </is>
       </c>
-      <c r="O35" s="211" t="inlineStr">
-        <is>
-          <t>│</t>
-        </is>
-      </c>
+      <c r="O35" s="211" t="n"/>
       <c r="P35" s="72" t="n"/>
       <c r="Q35" s="62" t="inlineStr">
         <is>
@@ -7047,7 +6968,7 @@
       </c>
       <c r="X35" s="219" t="inlineStr">
         <is>
-          <t>｜入学説明会</t>
+          <t>入学説明会</t>
         </is>
       </c>
       <c r="Y35" s="38" t="n"/>
@@ -7132,11 +7053,7 @@
       <c r="N36" s="52" t="n">
         <v>17</v>
       </c>
-      <c r="O36" s="227" t="inlineStr">
-        <is>
-          <t>│</t>
-        </is>
-      </c>
+      <c r="O36" s="227" t="n"/>
       <c r="P36" s="53" t="n"/>
       <c r="Q36" s="65" t="n">
         <v>17</v>
@@ -7157,7 +7074,7 @@
       </c>
       <c r="X36" s="206" t="inlineStr">
         <is>
-          <t>｜</t>
+          <t>期末テスト</t>
         </is>
       </c>
       <c r="Y36" s="76" t="n"/>
@@ -7237,11 +7154,7 @@
           <t>火</t>
         </is>
       </c>
-      <c r="O37" s="211" t="inlineStr">
-        <is>
-          <t>│</t>
-        </is>
-      </c>
+      <c r="O37" s="211" t="n"/>
       <c r="P37" s="38" t="n"/>
       <c r="Q37" s="62" t="inlineStr">
         <is>
@@ -7262,11 +7175,7 @@
           <t>水</t>
         </is>
       </c>
-      <c r="X37" s="325" t="inlineStr">
-        <is>
-          <t>↓</t>
-        </is>
-      </c>
+      <c r="X37" s="325" t="n"/>
       <c r="Y37" s="38" t="n"/>
       <c r="Z37" s="57" t="inlineStr">
         <is>
@@ -7344,11 +7253,7 @@
       <c r="N38" s="52" t="n">
         <v>18</v>
       </c>
-      <c r="O38" s="227" t="inlineStr">
-        <is>
-          <t>│</t>
-        </is>
-      </c>
+      <c r="O38" s="227" t="n"/>
       <c r="P38" s="81" t="n"/>
       <c r="Q38" s="224" t="n">
         <v>18</v>
@@ -7440,11 +7345,7 @@
           <t>水</t>
         </is>
       </c>
-      <c r="O39" s="211" t="inlineStr">
-        <is>
-          <t>↓</t>
-        </is>
-      </c>
+      <c r="O39" s="211" t="n"/>
       <c r="P39" s="78" t="n"/>
       <c r="Q39" s="216" t="inlineStr">
         <is>
@@ -7951,7 +7852,7 @@
       </c>
       <c r="R44" s="245" t="inlineStr">
         <is>
-          <t>※ノー部活ウィーク</t>
+          <t>ノー部活ウィーク</t>
         </is>
       </c>
       <c r="S44" s="337" t="n"/>
@@ -8043,11 +7944,7 @@
           <t>火</t>
         </is>
       </c>
-      <c r="R45" s="276" t="inlineStr">
-        <is>
-          <t>│</t>
-        </is>
-      </c>
+      <c r="R45" s="276" t="n"/>
       <c r="S45" s="338" t="n"/>
       <c r="T45" s="62" t="inlineStr">
         <is>
@@ -8143,7 +8040,7 @@
       </c>
       <c r="R46" s="340" t="inlineStr">
         <is>
-          <t>│</t>
+          <t>ノー部活ウィーク</t>
         </is>
       </c>
       <c r="S46" s="341" t="n"/>
@@ -8510,7 +8407,7 @@
       </c>
       <c r="R50" s="234" t="inlineStr">
         <is>
-          <t>│</t>
+          <t>ノー部活ウィーク</t>
         </is>
       </c>
       <c r="S50" s="103" t="inlineStr">
@@ -8602,7 +8499,7 @@
       </c>
       <c r="I51" s="346" t="inlineStr">
         <is>
-          <t>｜保護者試食会</t>
+          <t>保護者試食会</t>
         </is>
       </c>
       <c r="J51" s="58" t="n"/>
@@ -8627,7 +8524,7 @@
       </c>
       <c r="R51" s="346" t="inlineStr">
         <is>
-          <t>│　　　　　専修合同説明会</t>
+          <t>専修合同説明会</t>
         </is>
       </c>
       <c r="S51" s="92" t="n"/>
@@ -8706,7 +8603,7 @@
       </c>
       <c r="I52" s="234" t="inlineStr">
         <is>
-          <t>｜</t>
+          <t>期末テスト</t>
         </is>
       </c>
       <c r="J52" s="96" t="n"/>
@@ -8723,11 +8620,7 @@
       <c r="Q52" s="224" t="n">
         <v>25</v>
       </c>
-      <c r="R52" s="291" t="inlineStr">
-        <is>
-          <t>│</t>
-        </is>
-      </c>
+      <c r="R52" s="291" t="n"/>
       <c r="S52" s="250" t="n"/>
       <c r="T52" s="65" t="n">
         <v>25</v>
@@ -8808,11 +8701,7 @@
           <t>金</t>
         </is>
       </c>
-      <c r="I53" s="346" t="inlineStr">
-        <is>
-          <t>｜</t>
-        </is>
-      </c>
+      <c r="I53" s="346" t="n"/>
       <c r="J53" s="61" t="n"/>
       <c r="K53" s="216" t="inlineStr">
         <is>
@@ -8833,11 +8722,7 @@
           <t>土</t>
         </is>
       </c>
-      <c r="R53" s="349" t="inlineStr">
-        <is>
-          <t>│</t>
-        </is>
-      </c>
+      <c r="R53" s="349" t="n"/>
       <c r="S53" s="345" t="n"/>
       <c r="T53" s="62" t="inlineStr">
         <is>
@@ -8911,11 +8796,7 @@
       <c r="H54" s="221" t="n">
         <v>26</v>
       </c>
-      <c r="I54" s="291" t="inlineStr">
-        <is>
-          <t>｜</t>
-        </is>
-      </c>
+      <c r="I54" s="291" t="n"/>
       <c r="J54" s="209" t="n"/>
       <c r="K54" s="65" t="n">
         <v>26</v>
@@ -8930,11 +8811,7 @@
       <c r="Q54" s="207" t="n">
         <v>26</v>
       </c>
-      <c r="R54" s="255" t="inlineStr">
-        <is>
-          <t>│</t>
-        </is>
-      </c>
+      <c r="R54" s="255" t="n"/>
       <c r="S54" s="244" t="n"/>
       <c r="T54" s="65" t="n">
         <v>26</v>
@@ -9006,11 +8883,7 @@
           <t>土</t>
         </is>
       </c>
-      <c r="I55" s="349" t="inlineStr">
-        <is>
-          <t>｜</t>
-        </is>
-      </c>
+      <c r="I55" s="349" t="n"/>
       <c r="J55" s="218" t="n"/>
       <c r="K55" s="62" t="inlineStr">
         <is>
@@ -9031,11 +8904,7 @@
           <t>日</t>
         </is>
       </c>
-      <c r="R55" s="232" t="inlineStr">
-        <is>
-          <t>↓</t>
-        </is>
-      </c>
+      <c r="R55" s="232" t="n"/>
       <c r="S55" s="250" t="n"/>
       <c r="T55" s="62" t="inlineStr">
         <is>
@@ -9113,11 +8982,7 @@
       <c r="H56" s="207" t="n">
         <v>27</v>
       </c>
-      <c r="I56" s="255" t="inlineStr">
-        <is>
-          <t>｜</t>
-        </is>
-      </c>
+      <c r="I56" s="255" t="n"/>
       <c r="J56" s="209" t="n"/>
       <c r="K56" s="65" t="n">
         <v>27</v>
@@ -9212,11 +9077,7 @@
           <t>日</t>
         </is>
       </c>
-      <c r="I57" s="232" t="inlineStr">
-        <is>
-          <t>｜</t>
-        </is>
-      </c>
+      <c r="I57" s="232" t="n"/>
       <c r="J57" s="218" t="n"/>
       <c r="K57" s="62" t="inlineStr">
         <is>
@@ -9239,7 +9100,7 @@
       </c>
       <c r="R57" s="211" t="inlineStr">
         <is>
-          <t>｜ノー部活デー</t>
+          <t>ノー部活デー</t>
         </is>
       </c>
       <c r="S57" s="114" t="n"/>
@@ -9262,11 +9123,7 @@
           <t>月</t>
         </is>
       </c>
-      <c r="AA57" s="211" t="inlineStr">
-        <is>
-          <t>｜</t>
-        </is>
-      </c>
+      <c r="AA57" s="211" t="n"/>
       <c r="AB57" s="72" t="n"/>
       <c r="AC57" s="57" t="inlineStr">
         <is>
@@ -9313,7 +9170,7 @@
       </c>
       <c r="I58" s="206" t="inlineStr">
         <is>
-          <t>｜</t>
+          <t>期末テスト</t>
         </is>
       </c>
       <c r="J58" s="147" t="n"/>
@@ -9332,7 +9189,7 @@
       </c>
       <c r="R58" s="354" t="inlineStr">
         <is>
-          <t>｜</t>
+          <t>専修合同説明会</t>
         </is>
       </c>
       <c r="S58" s="66" t="n"/>
@@ -9355,7 +9212,7 @@
       </c>
       <c r="AA58" s="227" t="inlineStr">
         <is>
-          <t>｜</t>
+          <t>ノー部活ウィーク</t>
         </is>
       </c>
       <c r="AB58" s="53" t="n"/>
@@ -9402,11 +9259,7 @@
           <t>月</t>
         </is>
       </c>
-      <c r="I59" s="211" t="inlineStr">
-        <is>
-          <t>↓</t>
-        </is>
-      </c>
+      <c r="I59" s="211" t="n"/>
       <c r="J59" s="72" t="n"/>
       <c r="K59" s="57" t="inlineStr">
         <is>
@@ -9429,7 +9282,7 @@
       </c>
       <c r="R59" s="211" t="inlineStr">
         <is>
-          <t>↓　　　　　専修合同説明会</t>
+          <t>中間テスト</t>
         </is>
       </c>
       <c r="S59" s="50" t="n"/>
@@ -9452,11 +9305,7 @@
           <t>火</t>
         </is>
       </c>
-      <c r="AA59" s="211" t="inlineStr">
-        <is>
-          <t>｜</t>
-        </is>
-      </c>
+      <c r="AA59" s="211" t="n"/>
       <c r="AB59" s="38" t="n"/>
       <c r="AC59" s="57" t="inlineStr">
         <is>
@@ -9545,7 +9394,7 @@
       </c>
       <c r="AA60" s="227" t="inlineStr">
         <is>
-          <t>｜</t>
+          <t>ノー部活ウィーク</t>
         </is>
       </c>
       <c r="AB60" s="53" t="n"/>
@@ -9638,11 +9487,7 @@
           <t>水</t>
         </is>
       </c>
-      <c r="AA61" s="219" t="inlineStr">
-        <is>
-          <t>｜</t>
-        </is>
-      </c>
+      <c r="AA61" s="219" t="n"/>
       <c r="AB61" s="61" t="n"/>
       <c r="AC61" s="203" t="inlineStr">
         <is>
@@ -9673,9 +9518,9 @@
       <c r="B62" s="52" t="n">
         <v>30</v>
       </c>
-      <c r="C62" s="22" t="inlineStr">
-        <is>
-          <t>⑤⑥修学旅行・進路説明会(3年)</t>
+      <c r="C62" s="423" t="inlineStr">
+        <is>
+          <t>部活保護者会</t>
         </is>
       </c>
       <c r="D62" s="53" t="inlineStr">
@@ -9739,7 +9584,7 @@
       </c>
       <c r="AA62" s="210" t="inlineStr">
         <is>
-          <t>｜</t>
+          <t>ノー部活ウィーク</t>
         </is>
       </c>
       <c r="AB62" s="38" t="n"/>
@@ -9763,11 +9608,7 @@
           <t>金</t>
         </is>
       </c>
-      <c r="C63" s="44" t="inlineStr">
-        <is>
-          <t>部活保護者会</t>
-        </is>
-      </c>
+      <c r="C63" s="44" t="n"/>
       <c r="D63" s="43" t="n"/>
       <c r="E63" s="203" t="inlineStr">
         <is>
@@ -9827,11 +9668,7 @@
           <t>木</t>
         </is>
       </c>
-      <c r="AA63" s="364" t="inlineStr">
-        <is>
-          <t>｜</t>
-        </is>
-      </c>
+      <c r="AA63" s="364" t="n"/>
       <c r="AB63" s="37" t="n"/>
       <c r="AC63" s="351" t="inlineStr">
         <is>
@@ -10077,7 +9914,7 @@
       </c>
       <c r="F65" s="44" t="inlineStr">
         <is>
-          <t>｜ノー部活ウィーク</t>
+          <t>ノー部活ウィーク</t>
         </is>
       </c>
       <c r="G65" s="43" t="n"/>
@@ -10812,7 +10649,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D70"/>
+  <dimension ref="A1:D73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16.15"/>
   <cols>
     <col width="14" customWidth="1" style="201" min="1" max="1"/>
@@ -12009,37 +11846,58 @@
       </c>
     </row>
     <row r="66">
-      <c r="A66" t="inlineStr">
+      <c r="A66" s="0" t="inlineStr">
         <is>
           <t>学校の指示で修正した点</t>
         </is>
       </c>
     </row>
     <row r="67">
-      <c r="A67" t="inlineStr">
+      <c r="A67" s="0" t="inlineStr">
         <is>
           <t>・修学旅行(3年)を6/8(火)〜6/10(木)に変更。その週の健診（耳鼻科・歯科）は6/15〜6/17の同じ曜日へ移動。</t>
         </is>
       </c>
     </row>
     <row r="68">
-      <c r="A68" t="inlineStr">
+      <c r="A68" s="0" t="inlineStr">
         <is>
           <t>・修学旅行事前指導(3年)は出発前の6/7(月)へ移動（要確認）。心臓検診(1年)は6/11(金)のまま。</t>
         </is>
       </c>
     </row>
     <row r="69">
-      <c r="A69" t="inlineStr">
+      <c r="A69" s="0" t="inlineStr">
         <is>
           <t>・稲武野外学習(2年)と事前指導を5月から削除。7〜8月実施予定（日程未定）。</t>
         </is>
       </c>
     </row>
     <row r="70">
-      <c r="A70" t="inlineStr">
+      <c r="A70" s="0" t="inlineStr">
         <is>
           <t>・稲武野外学習説明会(2年)を6/22(火)へ移動（6月下旬で調整中）。</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="0" t="inlineStr">
+        <is>
+          <t>・日付をまたぐ行事は、矢印をやめて各日に同じ内容を書いた（土日・祝日には書かない）。</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="0" t="inlineStr">
+        <is>
+          <t>・修学旅行・進路説明会(3年)を4/30から5/6(木)の5・6限へ移動。木曜の研修（14:05〜）と時間が重なるため要調整。</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>・陸前高田市交流(2年)は令和9年度は実施しないため削除。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Remove parents' lunch tasting event from FY2027 plan
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FawjLRytv2ATkyFXeWDDqM
</commit_message>
<xml_diff>
--- a/令和9年度_年間計画（案）.xlsx
+++ b/令和9年度_年間計画（案）.xlsx
@@ -8497,11 +8497,7 @@
           <t>木</t>
         </is>
       </c>
-      <c r="I51" s="346" t="inlineStr">
-        <is>
-          <t>保護者試食会</t>
-        </is>
-      </c>
+      <c r="I51" s="346" t="n"/>
       <c r="J51" s="58" t="n"/>
       <c r="K51" s="203" t="inlineStr">
         <is>
@@ -10649,7 +10645,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D73"/>
+  <dimension ref="A1:D74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16.15"/>
   <cols>
     <col width="14" customWidth="1" style="201" min="1" max="1"/>
@@ -11895,9 +11891,16 @@
       </c>
     </row>
     <row r="73">
-      <c r="A73" t="inlineStr">
+      <c r="A73" s="0" t="inlineStr">
         <is>
           <t>・陸前高田市交流(2年)は令和9年度は実施しないため削除。</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>・保護者試食会は令和9年度は実施しないため削除。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Split briefings to 4/30 and 5/7; shorten grade 1-2 conference periods to 4 days
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FawjLRytv2ATkyFXeWDDqM
</commit_message>
<xml_diff>
--- a/令和9年度_年間計画（案）.xlsx
+++ b/令和9年度_年間計画（案）.xlsx
@@ -3986,7 +3986,7 @@
       </c>
       <c r="I10" s="242" t="inlineStr">
         <is>
-          <t>教育相談（全学年）</t>
+          <t>教育相談（3年）</t>
         </is>
       </c>
       <c r="K10" s="207" t="n">
@@ -4672,7 +4672,7 @@
       </c>
       <c r="F15" s="264" t="inlineStr">
         <is>
-          <t>新体力テスト準備・⑤⑥修学旅行・進路説明会(3年)</t>
+          <t>新体力テスト準備</t>
         </is>
       </c>
       <c r="G15" s="61" t="n"/>
@@ -4879,7 +4879,7 @@
       </c>
       <c r="AA16" s="227" t="inlineStr">
         <is>
-          <t>保護者会(全)</t>
+          <t>保護者会(3年)</t>
         </is>
       </c>
       <c r="AB16" s="53" t="n"/>
@@ -4979,7 +4979,11 @@
           <t>金</t>
         </is>
       </c>
-      <c r="F17" s="13" t="n"/>
+      <c r="F17" s="13" t="inlineStr">
+        <is>
+          <t>⑤⑥修学旅行説明会(3年)</t>
+        </is>
+      </c>
       <c r="G17" s="69" t="n"/>
       <c r="H17" s="62" t="inlineStr">
         <is>
@@ -5376,7 +5380,7 @@
       </c>
       <c r="L20" s="211" t="inlineStr">
         <is>
-          <t>保護者会（全）</t>
+          <t>保護者会（3年）</t>
         </is>
       </c>
       <c r="M20" s="53" t="n"/>
@@ -6760,7 +6764,7 @@
       </c>
       <c r="X33" s="211" t="inlineStr">
         <is>
-          <t>教育相談(1・2年)・ノー部活ウィーク</t>
+          <t>ノー部活ウィーク</t>
         </is>
       </c>
       <c r="Y33" s="72" t="n"/>
@@ -9516,7 +9520,7 @@
       </c>
       <c r="C62" s="423" t="inlineStr">
         <is>
-          <t>部活保護者会</t>
+          <t>⑤⑥進路説明会(3年)</t>
         </is>
       </c>
       <c r="D62" s="53" t="inlineStr">
@@ -9604,7 +9608,11 @@
           <t>金</t>
         </is>
       </c>
-      <c r="C63" s="44" t="n"/>
+      <c r="C63" s="44" t="inlineStr">
+        <is>
+          <t>部活保護者会</t>
+        </is>
+      </c>
       <c r="D63" s="43" t="n"/>
       <c r="E63" s="203" t="inlineStr">
         <is>
@@ -10645,7 +10653,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D74"/>
+  <dimension ref="A1:D76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16.15"/>
   <cols>
     <col width="14" customWidth="1" style="201" min="1" max="1"/>
@@ -11898,9 +11906,23 @@
       </c>
     </row>
     <row r="74">
-      <c r="A74" t="inlineStr">
+      <c r="A74" s="0" t="inlineStr">
         <is>
           <t>・保護者試食会は令和9年度は実施しないため削除。</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>・進路説明会(3年)は4/30(金)⑤⑥のまま。修学旅行説明会(3年)は5/7(金)⑤⑥。</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>・保護者会・教育相談の期間は、1・2年は木曜を含む4日間（最終日は3年のみ）：教育相談5/31〜6/3、保護者会7/5〜7/8、教育相談11/9〜11/12、保護者会12/1〜12/6。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Set physical fitness test schedule (5/7 prep, 5/10, 5/11 backup)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FawjLRytv2ATkyFXeWDDqM
</commit_message>
<xml_diff>
--- a/令和9年度_年間計画（案）.xlsx
+++ b/令和9年度_年間計画（案）.xlsx
@@ -1189,7 +1189,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="31" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="424">
+  <cellXfs count="427">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <protection locked="0" hidden="0"/>
     </xf>
@@ -2409,6 +2409,15 @@
     </xf>
     <xf numFmtId="1" fontId="33" fillId="0" borderId="26" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="2">
       <alignment horizontal="justify" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="33" fillId="0" borderId="26" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="2">
+      <alignment vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="33" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="2">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="33" fillId="0" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="2">
+      <alignment vertical="center" shrinkToFit="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="4">
@@ -4530,7 +4539,7 @@
       <c r="E14" s="52" t="n">
         <v>6</v>
       </c>
-      <c r="F14" s="262" t="inlineStr">
+      <c r="F14" s="424" t="inlineStr">
         <is>
           <t>本時間割</t>
         </is>
@@ -4670,11 +4679,7 @@
           <t>木</t>
         </is>
       </c>
-      <c r="F15" s="264" t="inlineStr">
-        <is>
-          <t>新体力テスト準備</t>
-        </is>
-      </c>
+      <c r="F15" s="425" t="n"/>
       <c r="G15" s="61" t="n"/>
       <c r="H15" s="216" t="inlineStr">
         <is>
@@ -4810,9 +4815,9 @@
       <c r="E16" s="52" t="n">
         <v>7</v>
       </c>
-      <c r="F16" s="263" t="inlineStr">
-        <is>
-          <t>新体力テスト</t>
+      <c r="F16" s="416" t="inlineStr">
+        <is>
+          <t>新体力テスト準備</t>
         </is>
       </c>
       <c r="G16" s="38" t="inlineStr">
@@ -4979,7 +4984,7 @@
           <t>金</t>
         </is>
       </c>
-      <c r="F17" s="13" t="inlineStr">
+      <c r="F17" s="425" t="inlineStr">
         <is>
           <t>⑤⑥修学旅行説明会(3年)</t>
         </is>
@@ -5593,9 +5598,9 @@
       <c r="E22" s="65" t="n">
         <v>10</v>
       </c>
-      <c r="F22" s="254" t="inlineStr">
-        <is>
-          <t>新体力テスト予備日</t>
+      <c r="F22" s="413" t="inlineStr">
+        <is>
+          <t>新体力テスト</t>
         </is>
       </c>
       <c r="G22" s="147" t="n"/>
@@ -5691,7 +5696,7 @@
           <t>月</t>
         </is>
       </c>
-      <c r="F23" s="68" t="n"/>
+      <c r="F23" s="414" t="n"/>
       <c r="G23" s="72" t="n"/>
       <c r="H23" s="57" t="inlineStr">
         <is>
@@ -5785,7 +5790,11 @@
       <c r="E24" s="65" t="n">
         <v>11</v>
       </c>
-      <c r="F24" s="16" t="n"/>
+      <c r="F24" s="413" t="inlineStr">
+        <is>
+          <t>新体力テスト予備日</t>
+        </is>
+      </c>
       <c r="G24" s="91" t="n"/>
       <c r="H24" s="52" t="n">
         <v>11</v>
@@ -5883,7 +5892,7 @@
           <t>火</t>
         </is>
       </c>
-      <c r="F25" s="134" t="n"/>
+      <c r="F25" s="426" t="n"/>
       <c r="G25" s="38" t="n"/>
       <c r="H25" s="57" t="inlineStr">
         <is>
@@ -10653,7 +10662,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D76"/>
+  <dimension ref="A1:D77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16.15"/>
   <cols>
     <col width="14" customWidth="1" style="201" min="1" max="1"/>
@@ -11913,16 +11922,23 @@
       </c>
     </row>
     <row r="75">
-      <c r="A75" t="inlineStr">
+      <c r="A75" s="0" t="inlineStr">
         <is>
           <t>・進路説明会(3年)は4/30(金)⑤⑥のまま。修学旅行説明会(3年)は5/7(金)⑤⑥。</t>
         </is>
       </c>
     </row>
     <row r="76">
-      <c r="A76" t="inlineStr">
+      <c r="A76" s="0" t="inlineStr">
         <is>
           <t>・保護者会・教育相談の期間は、1・2年は木曜を含む4日間（最終日は3年のみ）：教育相談5/31〜6/3、保護者会7/5〜7/8、教育相談11/9〜11/12、保護者会12/1〜12/6。</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>・新体力テスト：5/7(金)準備、5/10(月)実施、5/11(火)予備日。修学旅行説明会(3年)は5/7(金)⑤⑥。日程確定のため黒字にした。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Move adolescence seminar to 9/10
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FawjLRytv2ATkyFXeWDDqM
</commit_message>
<xml_diff>
--- a/令和9年度_年間計画（案）.xlsx
+++ b/令和9年度_年間計画（案）.xlsx
@@ -3696,11 +3696,7 @@
       <c r="Q8" s="65" t="n">
         <v>3</v>
       </c>
-      <c r="R8" s="206" t="inlineStr">
-        <is>
-          <t>思春期セミナー（3年）</t>
-        </is>
-      </c>
+      <c r="R8" s="206" t="n"/>
       <c r="S8" s="50" t="inlineStr">
         <is>
           <t>委</t>
@@ -5630,7 +5626,11 @@
       <c r="Q22" s="65" t="n">
         <v>10</v>
       </c>
-      <c r="R22" s="64" t="n"/>
+      <c r="R22" s="206" t="inlineStr">
+        <is>
+          <t>思春期セミナー（3年）</t>
+        </is>
+      </c>
       <c r="S22" s="73" t="n"/>
       <c r="T22" s="207" t="n">
         <v>10</v>
@@ -10662,7 +10662,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D77"/>
+  <dimension ref="A1:D78"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16.15"/>
   <cols>
     <col width="14" customWidth="1" style="201" min="1" max="1"/>
@@ -11936,9 +11936,16 @@
       </c>
     </row>
     <row r="77">
-      <c r="A77" t="inlineStr">
+      <c r="A77" s="0" t="inlineStr">
         <is>
           <t>・新体力テスト：5/7(金)準備、5/10(月)実施、5/11(火)予備日。修学旅行説明会(3年)は5/7(金)⑤⑥。日程確定のため黒字にした。</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>・思春期セミナー(3年)を9/10(金)へ移動。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Apply review fixes and mark 35 Thursday training sessions in FY2027 plan
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FawjLRytv2ATkyFXeWDDqM
</commit_message>
<xml_diff>
--- a/令和9年度_年間計画（案）.xlsx
+++ b/令和9年度_年間計画（案）.xlsx
@@ -263,7 +263,7 @@
       <sz val="12"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -273,6 +273,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF92D050"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFF99"/>
       </patternFill>
     </fill>
   </fills>
@@ -1189,7 +1194,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="31" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="427">
+  <cellXfs count="428">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <protection locked="0" hidden="0"/>
     </xf>
@@ -2418,6 +2423,9 @@
     </xf>
     <xf numFmtId="1" fontId="33" fillId="0" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="2">
       <alignment vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="34" fillId="3" borderId="26" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="2">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="4">
@@ -3091,7 +3099,7 @@
       </c>
       <c r="D4" s="140" t="inlineStr">
         <is>
-          <t>学2</t>
+          <t>職1</t>
         </is>
       </c>
       <c r="E4" s="203" t="n">
@@ -3203,7 +3211,7 @@
       <c r="C5" s="56" t="n"/>
       <c r="D5" s="61" t="inlineStr">
         <is>
-          <t>教･部活</t>
+          <t>学1</t>
         </is>
       </c>
       <c r="E5" s="203" t="inlineStr">
@@ -3232,7 +3240,8 @@
       <c r="L5" s="167" t="n"/>
       <c r="M5" s="38" t="inlineStr">
         <is>
-          <t>職6</t>
+          <t>職6
+研10</t>
         </is>
       </c>
       <c r="N5" s="216" t="inlineStr">
@@ -3360,7 +3369,11 @@
           <t>ノー部活デー</t>
         </is>
       </c>
-      <c r="D6" s="90" t="n"/>
+      <c r="D6" s="90" t="inlineStr">
+        <is>
+          <t>学2</t>
+        </is>
+      </c>
       <c r="E6" s="221" t="n">
         <v>2</v>
       </c>
@@ -3407,7 +3420,11 @@
       <c r="W6" s="52" t="n">
         <v>2</v>
       </c>
-      <c r="X6" s="64" t="n"/>
+      <c r="X6" s="64" t="inlineStr">
+        <is>
+          <t>文化祭(音楽発表会)準備</t>
+        </is>
+      </c>
       <c r="Y6" s="38" t="n"/>
       <c r="Z6" s="52" t="n">
         <v>2</v>
@@ -3440,7 +3457,11 @@
           <t>卒業式準備</t>
         </is>
       </c>
-      <c r="AK6" s="165" t="n"/>
+      <c r="AK6" s="165" t="inlineStr">
+        <is>
+          <t>研32</t>
+        </is>
+      </c>
       <c r="AL6" s="31" t="n"/>
       <c r="AM6" s="32" t="n"/>
       <c r="AN6" s="163" t="inlineStr">
@@ -3507,7 +3528,11 @@
         </is>
       </c>
       <c r="C7" s="68" t="n"/>
-      <c r="D7" s="72" t="n"/>
+      <c r="D7" s="72" t="inlineStr">
+        <is>
+          <t>教･部活</t>
+        </is>
+      </c>
       <c r="E7" s="203" t="inlineStr">
         <is>
           <t>日</t>
@@ -3548,7 +3573,8 @@
       <c r="R7" s="13" t="n"/>
       <c r="S7" s="92" t="inlineStr">
         <is>
-          <t>現4</t>
+          <t>現4
+研12</t>
         </is>
       </c>
       <c r="T7" s="216" t="inlineStr">
@@ -3900,7 +3926,11 @@
           <t>【公立推薦･特色入試】</t>
         </is>
       </c>
-      <c r="AH9" s="38" t="n"/>
+      <c r="AH9" s="38" t="inlineStr">
+        <is>
+          <t>研28</t>
+        </is>
+      </c>
       <c r="AI9" s="57" t="inlineStr">
         <is>
           <t>金</t>
@@ -4017,11 +4047,7 @@
       <c r="W10" s="52" t="n">
         <v>4</v>
       </c>
-      <c r="X10" s="245" t="inlineStr">
-        <is>
-          <t>※文化祭(音楽発表会)準備</t>
-        </is>
-      </c>
+      <c r="X10" s="245" t="n"/>
       <c r="Y10" s="38" t="inlineStr">
         <is>
           <t>運9</t>
@@ -4174,7 +4200,11 @@
           <t>文化祭（音楽発表会）</t>
         </is>
       </c>
-      <c r="Y11" s="38" t="n"/>
+      <c r="Y11" s="38" t="inlineStr">
+        <is>
+          <t>研19</t>
+        </is>
+      </c>
       <c r="Z11" s="203" t="inlineStr">
         <is>
           <t>土</t>
@@ -4676,7 +4706,11 @@
         </is>
       </c>
       <c r="F15" s="425" t="n"/>
-      <c r="G15" s="61" t="n"/>
+      <c r="G15" s="61" t="inlineStr">
+        <is>
+          <t>研4</t>
+        </is>
+      </c>
       <c r="H15" s="216" t="inlineStr">
         <is>
           <t>日</t>
@@ -5265,7 +5299,8 @@
         <is>
           <t>努･採
 運2
-職2</t>
+職2
+研1</t>
         </is>
       </c>
       <c r="E19" s="203" t="inlineStr">
@@ -5514,7 +5549,8 @@
       <c r="R21" s="68" t="n"/>
       <c r="S21" s="137" t="inlineStr">
         <is>
-          <t>学8</t>
+          <t>学8
+研13</t>
         </is>
       </c>
       <c r="T21" s="216" t="inlineStr">
@@ -5543,7 +5579,8 @@
       <c r="AA21" s="68" t="n"/>
       <c r="AB21" s="38" t="inlineStr">
         <is>
-          <t>進4</t>
+          <t>進4
+研22</t>
         </is>
       </c>
       <c r="AC21" s="203" t="inlineStr">
@@ -5577,7 +5614,8 @@
       <c r="AK21" s="0" t="inlineStr">
         <is>
           <t>職11
-編1</t>
+編1
+研33</t>
         </is>
       </c>
       <c r="AL21" s="31" t="n"/>
@@ -5768,7 +5806,11 @@
         </is>
       </c>
       <c r="AG23" s="84" t="n"/>
-      <c r="AH23" s="131" t="n"/>
+      <c r="AH23" s="131" t="inlineStr">
+        <is>
+          <t>研29</t>
+        </is>
+      </c>
       <c r="AI23" s="57" t="inlineStr">
         <is>
           <t>金</t>
@@ -5846,11 +5888,7 @@
         <v>11</v>
       </c>
       <c r="AA24" s="208" t="n"/>
-      <c r="AB24" s="209" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
+      <c r="AB24" s="209" t="n"/>
       <c r="AC24" s="52" t="n">
         <v>11</v>
       </c>
@@ -6072,11 +6110,7 @@
         <v>12</v>
       </c>
       <c r="AG26" s="217" t="n"/>
-      <c r="AH26" s="286" t="inlineStr">
-        <is>
-          <t>委</t>
-        </is>
-      </c>
+      <c r="AH26" s="286" t="n"/>
       <c r="AI26" s="221" t="n">
         <v>12</v>
       </c>
@@ -6263,7 +6297,11 @@
           <t>保護者会(3年)</t>
         </is>
       </c>
-      <c r="AE28" s="53" t="n"/>
+      <c r="AE28" s="53" t="inlineStr">
+        <is>
+          <t>研25</t>
+        </is>
+      </c>
       <c r="AF28" s="221" t="n">
         <v>13</v>
       </c>
@@ -6311,7 +6349,8 @@
       <c r="F29" s="127" t="n"/>
       <c r="G29" s="59" t="inlineStr">
         <is>
-          <t>職4</t>
+          <t>職4
+研5</t>
         </is>
       </c>
       <c r="H29" s="313" t="inlineStr">
@@ -6551,7 +6590,11 @@
         </is>
       </c>
       <c r="U31" s="18" t="n"/>
-      <c r="V31" s="61" t="n"/>
+      <c r="V31" s="61" t="inlineStr">
+        <is>
+          <t>研16</t>
+        </is>
+      </c>
       <c r="W31" s="216" t="inlineStr">
         <is>
           <t>日</t>
@@ -6579,7 +6622,11 @@
         </is>
       </c>
       <c r="AG31" s="18" t="n"/>
-      <c r="AH31" s="38" t="n"/>
+      <c r="AH31" s="38" t="inlineStr">
+        <is>
+          <t>委</t>
+        </is>
+      </c>
       <c r="AI31" s="57" t="inlineStr">
         <is>
           <t>火</t>
@@ -6626,12 +6673,12 @@
       <c r="K32" s="52" t="n">
         <v>15</v>
       </c>
-      <c r="L32" s="227" t="inlineStr">
-        <is>
-          <t>大掃除</t>
-        </is>
-      </c>
-      <c r="M32" s="53" t="n"/>
+      <c r="L32" s="227" t="n"/>
+      <c r="M32" s="53" t="inlineStr">
+        <is>
+          <t>研11</t>
+        </is>
+      </c>
       <c r="N32" s="207" t="n">
         <v>15</v>
       </c>
@@ -6717,7 +6764,8 @@
         <is>
           <t>運3
 不
-進1</t>
+進1
+研2</t>
         </is>
       </c>
       <c r="E33" s="203" t="inlineStr">
@@ -6837,7 +6885,11 @@
       <c r="K34" s="52" t="n">
         <v>16</v>
       </c>
-      <c r="L34" s="86" t="n"/>
+      <c r="L34" s="86" t="inlineStr">
+        <is>
+          <t>大掃除</t>
+        </is>
+      </c>
       <c r="M34" s="53" t="n"/>
       <c r="N34" s="65" t="n">
         <v>16</v>
@@ -6964,7 +7016,8 @@
       <c r="R35" s="18" t="n"/>
       <c r="S35" s="50" t="inlineStr">
         <is>
-          <t>教</t>
+          <t>教
+研14</t>
         </is>
       </c>
       <c r="T35" s="216" t="inlineStr">
@@ -6993,7 +7046,8 @@
       <c r="AA35" s="68" t="n"/>
       <c r="AB35" s="72" t="inlineStr">
         <is>
-          <t>進学相談</t>
+          <t>進学相談
+研23</t>
         </is>
       </c>
       <c r="AC35" s="203" t="inlineStr">
@@ -7017,7 +7071,8 @@
       <c r="AJ35" s="322" t="n"/>
       <c r="AK35" s="0" t="inlineStr">
         <is>
-          <t>採</t>
+          <t>採
+研34</t>
         </is>
       </c>
       <c r="AL35" s="31" t="n"/>
@@ -7152,7 +7207,8 @@
       <c r="I37" s="70" t="n"/>
       <c r="J37" s="61" t="inlineStr">
         <is>
-          <t>運6</t>
+          <t>運6
+研8</t>
         </is>
       </c>
       <c r="K37" s="203" t="inlineStr">
@@ -7216,7 +7272,7 @@
       </c>
       <c r="AH37" s="61" t="inlineStr">
         <is>
-          <t>学12</t>
+          <t>研30</t>
         </is>
       </c>
       <c r="AI37" s="57" t="inlineStr">
@@ -7380,7 +7436,11 @@
         </is>
       </c>
       <c r="X39" s="77" t="n"/>
-      <c r="Y39" s="38" t="n"/>
+      <c r="Y39" s="38" t="inlineStr">
+        <is>
+          <t>研20</t>
+        </is>
+      </c>
       <c r="Z39" s="203" t="inlineStr">
         <is>
           <t>土</t>
@@ -7748,7 +7808,8 @@
       <c r="F43" s="84" t="n"/>
       <c r="G43" s="112" t="inlineStr">
         <is>
-          <t>現2</t>
+          <t>現2
+研6</t>
         </is>
       </c>
       <c r="H43" s="216" t="inlineStr">
@@ -7810,7 +7871,11 @@
           <t>【私立専修一般入試】</t>
         </is>
       </c>
-      <c r="AE43" s="38" t="n"/>
+      <c r="AE43" s="38" t="inlineStr">
+        <is>
+          <t>研26</t>
+        </is>
+      </c>
       <c r="AF43" s="203" t="inlineStr">
         <is>
           <t>日</t>
@@ -7873,7 +7938,11 @@
         <v>21</v>
       </c>
       <c r="U44" s="16" t="n"/>
-      <c r="V44" s="53" t="n"/>
+      <c r="V44" s="53" t="inlineStr">
+        <is>
+          <t>研17</t>
+        </is>
+      </c>
       <c r="W44" s="221" t="n">
         <v>21</v>
       </c>
@@ -7882,11 +7951,7 @@
       <c r="Z44" s="52" t="n">
         <v>21</v>
       </c>
-      <c r="AA44" s="227" t="inlineStr">
-        <is>
-          <t>大掃除</t>
-        </is>
-      </c>
+      <c r="AA44" s="227" t="n"/>
       <c r="AB44" s="53" t="n"/>
       <c r="AC44" s="52" t="n">
         <v>21</v>
@@ -7905,11 +7970,7 @@
       <c r="AI44" s="52" t="n">
         <v>21</v>
       </c>
-      <c r="AJ44" s="227" t="inlineStr">
-        <is>
-          <t>大掃除</t>
-        </is>
-      </c>
+      <c r="AJ44" s="227" t="n"/>
       <c r="AK44" s="73" t="n"/>
       <c r="AL44" s="31" t="n"/>
       <c r="AM44" s="32" t="n"/>
@@ -8032,7 +8093,7 @@
       <c r="H46" s="65" t="n">
         <v>22</v>
       </c>
-      <c r="I46" s="420" t="inlineStr">
+      <c r="I46" s="427" t="inlineStr">
         <is>
           <t>稲武野外学習説明会(2年)</t>
         </is>
@@ -8078,7 +8139,11 @@
       <c r="Z46" s="52" t="n">
         <v>22</v>
       </c>
-      <c r="AA46" s="54" t="n"/>
+      <c r="AA46" s="54" t="inlineStr">
+        <is>
+          <t>大掃除</t>
+        </is>
+      </c>
       <c r="AB46" s="53" t="n"/>
       <c r="AC46" s="221" t="n">
         <v>22</v>
@@ -8107,7 +8172,11 @@
         </is>
       </c>
       <c r="C47" s="80" t="n"/>
-      <c r="D47" s="85" t="n"/>
+      <c r="D47" s="85" t="inlineStr">
+        <is>
+          <t>研3</t>
+        </is>
+      </c>
       <c r="E47" s="203" t="inlineStr">
         <is>
           <t>土</t>
@@ -8281,8 +8350,16 @@
       <c r="AI48" s="52" t="n">
         <v>23</v>
       </c>
-      <c r="AJ48" s="108" t="n"/>
-      <c r="AK48" s="107" t="n"/>
+      <c r="AJ48" s="108" t="inlineStr">
+        <is>
+          <t>大掃除</t>
+        </is>
+      </c>
+      <c r="AK48" s="107" t="inlineStr">
+        <is>
+          <t>研35</t>
+        </is>
+      </c>
       <c r="AL48" s="31" t="n"/>
       <c r="AM48" s="32" t="n"/>
       <c r="BA48" s="377" t="n"/>
@@ -8355,7 +8432,11 @@
         </is>
       </c>
       <c r="AA49" s="68" t="n"/>
-      <c r="AB49" s="38" t="n"/>
+      <c r="AB49" s="38" t="inlineStr">
+        <is>
+          <t>研24</t>
+        </is>
+      </c>
       <c r="AC49" s="203" t="inlineStr">
         <is>
           <t>日</t>
@@ -8404,7 +8485,11 @@
           <t>期末テスト</t>
         </is>
       </c>
-      <c r="J50" s="104" t="n"/>
+      <c r="J50" s="104" t="inlineStr">
+        <is>
+          <t>研9</t>
+        </is>
+      </c>
       <c r="K50" s="221" t="n">
         <v>24</v>
       </c>
@@ -8578,7 +8663,8 @@
       </c>
       <c r="AH51" s="61" t="inlineStr">
         <is>
-          <t>教</t>
+          <t>教
+研31</t>
         </is>
       </c>
       <c r="AI51" s="57" t="inlineStr">
@@ -8748,7 +8834,8 @@
       <c r="X53" s="350" t="n"/>
       <c r="Y53" s="0" t="inlineStr">
         <is>
-          <t>学10</t>
+          <t>学10
+研21</t>
         </is>
       </c>
       <c r="Z53" s="203" t="inlineStr">
@@ -9078,7 +9165,8 @@
       </c>
       <c r="G57" s="38" t="inlineStr">
         <is>
-          <t>教科等研究部会</t>
+          <t>教科等研究部会
+研7</t>
         </is>
       </c>
       <c r="H57" s="216" t="inlineStr">
@@ -9140,7 +9228,11 @@
         </is>
       </c>
       <c r="AD57" s="77" t="n"/>
-      <c r="AE57" s="61" t="n"/>
+      <c r="AE57" s="61" t="inlineStr">
+        <is>
+          <t>研27</t>
+        </is>
+      </c>
       <c r="AF57" s="203" t="inlineStr">
         <is>
           <t>日</t>
@@ -9301,7 +9393,11 @@
         </is>
       </c>
       <c r="U59" s="13" t="n"/>
-      <c r="V59" s="38" t="n"/>
+      <c r="V59" s="38" t="inlineStr">
+        <is>
+          <t>研18</t>
+        </is>
+      </c>
       <c r="W59" s="216" t="inlineStr">
         <is>
           <t>日</t>
@@ -9659,7 +9755,8 @@
       <c r="R63" s="44" t="n"/>
       <c r="S63" s="43" t="inlineStr">
         <is>
-          <t>現5</t>
+          <t>現5
+研15</t>
         </is>
       </c>
       <c r="T63" s="237" t="inlineStr">
@@ -10662,7 +10759,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D78"/>
+  <dimension ref="A1:D84"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16.15"/>
   <cols>
     <col width="14" customWidth="1" style="201" min="1" max="1"/>
@@ -11943,9 +12040,51 @@
       </c>
     </row>
     <row r="78">
-      <c r="A78" t="inlineStr">
+      <c r="A78" s="0" t="inlineStr">
         <is>
           <t>・思春期セミナー(3年)を9/10(金)へ移動。</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="0" t="inlineStr">
+        <is>
+          <t>・大掃除は終業式・修了式の前日（7/16、12/22、3/23）に実施。</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="0" t="inlineStr">
+        <is>
+          <t>・文化祭(音楽発表会)準備を11/2(火)へ移動。</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="0" t="inlineStr">
+        <is>
+          <t>・稲武野外学習説明会(2年) 6/22は仮置き（黄色の網かけ）。</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="0" t="inlineStr">
+        <is>
+          <t>・4/1に職1・学1、4/2に学2・教･部活を補充。12/11(土)の「4」を削除、2/12(土)の「委」を2/14(月)へ、2/17の学12の重複を削除。</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="0" t="inlineStr">
+        <is>
+          <t>・3年：入学式の日(4/7)と修学旅行の翌日(6/11)は家庭学習にせず授業日とする（授業数カウントで反映）。</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="0" t="inlineStr">
+        <is>
+          <t>・研修は木曜の5限後(14:05〜14:55)に年35回（会議記号の列に「研1〜研35」）。教育相談・保護者会・修学旅行・体育大会の木曜（6/3、6/10、7/8、10/7、11/11、12/2）は研修なし。会議は内容を工夫して研修の型に合うものにする。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Move graduation ceremony to 3/7
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FawjLRytv2ATkyFXeWDDqM
</commit_message>
<xml_diff>
--- a/令和9年度_年間計画（案）.xlsx
+++ b/令和9年度_年間計画（案）.xlsx
@@ -3452,11 +3452,7 @@
       <c r="AI6" s="52" t="n">
         <v>2</v>
       </c>
-      <c r="AJ6" s="228" t="inlineStr">
-        <is>
-          <t>卒業式準備</t>
-        </is>
-      </c>
+      <c r="AJ6" s="228" t="n"/>
       <c r="AK6" s="165" t="inlineStr">
         <is>
           <t>研32</t>
@@ -3772,16 +3768,8 @@
       <c r="AI8" s="52" t="n">
         <v>3</v>
       </c>
-      <c r="AJ8" s="227" t="inlineStr">
-        <is>
-          <t>卒業式</t>
-        </is>
-      </c>
-      <c r="AK8" s="50" t="inlineStr">
-        <is>
-          <t>定</t>
-        </is>
-      </c>
+      <c r="AJ8" s="227" t="n"/>
+      <c r="AK8" s="50" t="n"/>
       <c r="AL8" s="31" t="n"/>
       <c r="AM8" s="32" t="n"/>
       <c r="AN8" s="152" t="inlineStr">
@@ -4783,7 +4771,11 @@
           <t>月</t>
         </is>
       </c>
-      <c r="AJ15" s="80" t="n"/>
+      <c r="AJ15" s="80" t="inlineStr">
+        <is>
+          <t>卒業式準備</t>
+        </is>
+      </c>
       <c r="AK15" s="50" t="n"/>
       <c r="AL15" s="31" t="n"/>
       <c r="AM15" s="32" t="n"/>
@@ -4949,11 +4941,14 @@
       </c>
       <c r="AJ16" s="253" t="inlineStr">
         <is>
-          <t>選挙管理委員会
-　　　▼小中連絡会(汐路)</t>
-        </is>
-      </c>
-      <c r="AK16" s="73" t="n"/>
+          <t>卒業式</t>
+        </is>
+      </c>
+      <c r="AK16" s="73" t="inlineStr">
+        <is>
+          <t>定</t>
+        </is>
+      </c>
       <c r="AL16" s="31" t="n"/>
       <c r="AM16" s="32" t="n"/>
       <c r="AN16" s="152" t="inlineStr">
@@ -5117,7 +5112,7 @@
       </c>
       <c r="AJ17" s="270" t="inlineStr">
         <is>
-          <t>1･2年通知表（本）提出</t>
+          <t>選挙管理委員会・▼小中連絡会(汐路)・1･2年通知表（本）提出</t>
         </is>
       </c>
       <c r="AK17" s="50" t="n"/>
@@ -10759,7 +10754,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D84"/>
+  <dimension ref="A1:D85"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16.15"/>
   <cols>
     <col width="14" customWidth="1" style="201" min="1" max="1"/>
@@ -12088,6 +12083,13 @@
         </is>
       </c>
     </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>・卒業式を3/7(火)へ移動（定時退校日も移動）。卒業式準備は前日の3/6(月)。3/7の選挙管理委員会・小中連絡会(汐路)・1・2年通知表提出、3/6の公立一般合格発表との前後関係は要確認。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Place national achievement test provisionally on 4/15
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FawjLRytv2ATkyFXeWDDqM
</commit_message>
<xml_diff>
--- a/令和9年度_年間計画（案）.xlsx
+++ b/令和9年度_年間計画（案）.xlsx
@@ -6642,7 +6642,11 @@
       <c r="B32" s="65" t="n">
         <v>15</v>
       </c>
-      <c r="C32" s="16" t="n"/>
+      <c r="C32" s="427" t="inlineStr">
+        <is>
+          <t>全国学調(国･数･質)※4/13〜16で調整</t>
+        </is>
+      </c>
       <c r="D32" s="53" t="inlineStr">
         <is>
           <t>職3
@@ -8070,11 +8074,7 @@
       <c r="B46" s="65" t="n">
         <v>22</v>
       </c>
-      <c r="C46" s="390" t="inlineStr">
-        <is>
-          <t>全国学調(国･数･英3技能･質)</t>
-        </is>
-      </c>
+      <c r="C46" s="390" t="n"/>
       <c r="D46" s="53" t="inlineStr">
         <is>
           <t>学4</t>
@@ -10754,7 +10754,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D85"/>
+  <dimension ref="A1:D86"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16.15"/>
   <cols>
     <col width="14" customWidth="1" style="201" min="1" max="1"/>
@@ -12084,9 +12084,16 @@
       </c>
     </row>
     <row r="85">
-      <c r="A85" t="inlineStr">
+      <c r="A85" s="0" t="inlineStr">
         <is>
           <t>・卒業式を3/7(火)へ移動（定時退校日も移動）。卒業式準備は前日の3/6(月)。3/7の選挙管理委員会・小中連絡会(汐路)・1・2年通知表提出、3/6の公立一般合格発表との前後関係は要確認。</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>・全国学調は国・数・質問紙の3時間。4/13〜4/16のいずれかで、4/15(木)に仮置き（黄色の網かけ）。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Reschedule committee, March meetings, and term-end tests in FY2027 plan
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FawjLRytv2ATkyFXeWDDqM
</commit_message>
<xml_diff>
--- a/令和9年度_年間計画（案）.xlsx
+++ b/令和9年度_年間計画（案）.xlsx
@@ -1194,7 +1194,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="31" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="428">
+  <cellXfs count="429">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <protection locked="0" hidden="0"/>
     </xf>
@@ -2426,6 +2426,9 @@
     </xf>
     <xf numFmtId="1" fontId="34" fillId="3" borderId="26" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="2">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="35" fillId="0" borderId="26" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="2">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="4">
@@ -4627,7 +4630,7 @@
       <c r="AI14" s="52" t="n">
         <v>6</v>
       </c>
-      <c r="AJ14" s="234" t="inlineStr">
+      <c r="AJ14" s="428" t="inlineStr">
         <is>
           <t>【公立一般合格発表】</t>
         </is>
@@ -4931,11 +4934,7 @@
           <t>ノー部活ウィーク</t>
         </is>
       </c>
-      <c r="AH16" s="132" t="inlineStr">
-        <is>
-          <t>学保</t>
-        </is>
-      </c>
+      <c r="AH16" s="132" t="n"/>
       <c r="AI16" s="52" t="n">
         <v>7</v>
       </c>
@@ -5112,7 +5111,7 @@
       </c>
       <c r="AJ17" s="270" t="inlineStr">
         <is>
-          <t>選挙管理委員会・▼小中連絡会(汐路)・1･2年通知表（本）提出</t>
+          <t>1･2年通知表（本）提出</t>
         </is>
       </c>
       <c r="AK17" s="50" t="n"/>
@@ -5241,14 +5240,18 @@
       </c>
       <c r="AG18" s="262" t="inlineStr">
         <is>
-          <t>学年末テスト(１･２年)</t>
+          <t>ノー部活デー</t>
         </is>
       </c>
       <c r="AH18" s="144" t="n"/>
       <c r="AI18" s="52" t="n">
         <v>8</v>
       </c>
-      <c r="AJ18" s="54" t="n"/>
+      <c r="AJ18" s="54" t="inlineStr">
+        <is>
+          <t>選挙管理委員会</t>
+        </is>
+      </c>
       <c r="AK18" s="73" t="inlineStr">
         <is>
           <t>▼小中連絡会(陽明)</t>
@@ -5365,17 +5368,17 @@
           <t>火</t>
         </is>
       </c>
-      <c r="AG19" s="279" t="inlineStr">
-        <is>
-          <t>ノー部活デー</t>
-        </is>
-      </c>
+      <c r="AG19" s="279" t="n"/>
       <c r="AI19" s="57" t="inlineStr">
         <is>
           <t>水</t>
         </is>
       </c>
-      <c r="AJ19" s="143" t="n"/>
+      <c r="AJ19" s="143" t="inlineStr">
+        <is>
+          <t>▼小中連絡会(汐路)</t>
+        </is>
+      </c>
       <c r="AK19" s="50" t="n"/>
       <c r="AL19" s="31" t="n"/>
       <c r="AM19" s="32" t="n"/>
@@ -5466,7 +5469,7 @@
       </c>
       <c r="AG20" s="276" t="inlineStr">
         <is>
-          <t>学年末テスト(１･２年)</t>
+          <t>ノー部活デー</t>
         </is>
       </c>
       <c r="AH20" s="141" t="n"/>
@@ -5480,8 +5483,7 @@
       </c>
       <c r="AK20" s="0" t="inlineStr">
         <is>
-          <t>委
-進認</t>
+          <t>進認</t>
         </is>
       </c>
       <c r="AL20" s="31" t="n"/>
@@ -5590,11 +5592,7 @@
           <t>水</t>
         </is>
       </c>
-      <c r="AG21" s="211" t="inlineStr">
-        <is>
-          <t>ノー部活デー</t>
-        </is>
-      </c>
+      <c r="AG21" s="211" t="n"/>
       <c r="AH21" s="38" t="n"/>
       <c r="AI21" s="57" t="inlineStr">
         <is>
@@ -5696,11 +5694,7 @@
       <c r="AF22" s="52" t="n">
         <v>10</v>
       </c>
-      <c r="AG22" s="206" t="inlineStr">
-        <is>
-          <t>学年末テスト(１･２年)</t>
-        </is>
-      </c>
+      <c r="AG22" s="206" t="n"/>
       <c r="AH22" s="76" t="inlineStr">
         <is>
           <t>全反</t>
@@ -5710,7 +5704,11 @@
         <v>10</v>
       </c>
       <c r="AJ22" s="118" t="n"/>
-      <c r="AK22" s="139" t="n"/>
+      <c r="AK22" s="139" t="inlineStr">
+        <is>
+          <t>委</t>
+        </is>
+      </c>
       <c r="AL22" s="31" t="n"/>
       <c r="AM22" s="32" t="n"/>
       <c r="BA22" s="377" t="n"/>
@@ -6918,7 +6916,7 @@
       </c>
       <c r="X34" s="211" t="inlineStr">
         <is>
-          <t>期末テスト</t>
+          <t>入学説明会</t>
         </is>
       </c>
       <c r="Y34" s="53" t="n"/>
@@ -7031,11 +7029,7 @@
           <t>火</t>
         </is>
       </c>
-      <c r="X35" s="219" t="inlineStr">
-        <is>
-          <t>入学説明会</t>
-        </is>
-      </c>
+      <c r="X35" s="219" t="n"/>
       <c r="Y35" s="38" t="n"/>
       <c r="Z35" s="57" t="inlineStr">
         <is>
@@ -7164,12 +7158,13 @@
       </c>
       <c r="AG36" s="324" t="inlineStr">
         <is>
-          <t>学年保護者会(1年)</t>
+          <t>学年末テスト(１･２年)</t>
         </is>
       </c>
       <c r="AH36" s="119" t="inlineStr">
         <is>
           <t>学12
+学保
 ▼ＡＥＴ離任式</t>
         </is>
       </c>
@@ -7266,7 +7261,7 @@
       </c>
       <c r="AG37" s="276" t="inlineStr">
         <is>
-          <t>【定時制合格発表】</t>
+          <t>学年保護者会(1年)・【定時制合格発表】</t>
         </is>
       </c>
       <c r="AH37" s="61" t="inlineStr">
@@ -7344,7 +7339,11 @@
       <c r="W38" s="52" t="n">
         <v>18</v>
       </c>
-      <c r="X38" s="88" t="n"/>
+      <c r="X38" s="88" t="inlineStr">
+        <is>
+          <t>期末テスト</t>
+        </is>
+      </c>
       <c r="Y38" s="53" t="inlineStr">
         <is>
           <t>進3</t>
@@ -7363,7 +7362,11 @@
       <c r="AF38" s="52" t="n">
         <v>18</v>
       </c>
-      <c r="AG38" s="22" t="n"/>
+      <c r="AG38" s="22" t="inlineStr">
+        <is>
+          <t>学年末テスト(１･２年)</t>
+        </is>
+      </c>
       <c r="AH38" s="38" t="inlineStr">
         <is>
           <t>3年通知表(仮)提出</t>
@@ -10754,7 +10757,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D86"/>
+  <dimension ref="A1:D91"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16.15"/>
   <cols>
     <col width="14" customWidth="1" style="201" min="1" max="1"/>
@@ -12091,9 +12094,44 @@
       </c>
     </row>
     <row r="86">
-      <c r="A86" t="inlineStr">
+      <c r="A86" s="0" t="inlineStr">
         <is>
           <t>・全国学調は国・数・質問紙の3時間。4/13〜4/16のいずれかで、4/15(木)に仮置き（黄色の網かけ）。</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>・生徒委員会を3/9(木)から3/10(金)へ移動。</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>・選挙管理委員会・小中連絡会(汐路)を卒業式翌日の3/8(水)へ移動。</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>・公立一般合格発表(3/6)は日程未定のため赤字。</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>・2学期期末テストを11/17(水)・11/18(木)へ移動（入学説明会は11/16のまま）。</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>・学年末テスト(1・2年)を2/17(木)・2/18(金)へ移動。学校保健委員会(学保)も2/17へ移動。2/8・2/9のノー部活デーは残している。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Make all conference periods 4 days for every grade
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FawjLRytv2ATkyFXeWDDqM
</commit_message>
<xml_diff>
--- a/令和9年度_年間計画（案）.xlsx
+++ b/令和9年度_年間計画（案）.xlsx
@@ -4012,7 +4012,7 @@
       </c>
       <c r="I10" s="242" t="inlineStr">
         <is>
-          <t>教育相談（3年）</t>
+          <t>ノー部活ウィーク</t>
         </is>
       </c>
       <c r="K10" s="207" t="n">
@@ -4147,11 +4147,7 @@
           <t>金</t>
         </is>
       </c>
-      <c r="I11" s="211" t="inlineStr">
-        <is>
-          <t>ノー部活ウィーク</t>
-        </is>
-      </c>
+      <c r="I11" s="211" t="n"/>
       <c r="J11" s="58" t="n"/>
       <c r="K11" s="216" t="inlineStr">
         <is>
@@ -4909,7 +4905,7 @@
       </c>
       <c r="AA16" s="227" t="inlineStr">
         <is>
-          <t>保護者会(3年)</t>
+          <t>通知表(仮)提出</t>
         </is>
       </c>
       <c r="AB16" s="53" t="n"/>
@@ -5072,11 +5068,7 @@
           <t>火</t>
         </is>
       </c>
-      <c r="AA17" s="211" t="inlineStr">
-        <is>
-          <t>通知表(仮)提出</t>
-        </is>
-      </c>
+      <c r="AA17" s="211" t="n"/>
       <c r="AB17" s="38" t="n"/>
       <c r="AC17" s="57" t="inlineStr">
         <is>
@@ -5412,11 +5404,7 @@
       <c r="K20" s="52" t="n">
         <v>9</v>
       </c>
-      <c r="L20" s="211" t="inlineStr">
-        <is>
-          <t>保護者会（3年）</t>
-        </is>
-      </c>
+      <c r="L20" s="211" t="n"/>
       <c r="M20" s="53" t="n"/>
       <c r="N20" s="52" t="n">
         <v>9</v>
@@ -6704,7 +6692,7 @@
       </c>
       <c r="X32" s="206" t="inlineStr">
         <is>
-          <t>保護者会(3年)</t>
+          <t>ノー部活ウィーク</t>
         </is>
       </c>
       <c r="Y32" s="147" t="n"/>
@@ -6816,11 +6804,7 @@
           <t>月</t>
         </is>
       </c>
-      <c r="X33" s="211" t="inlineStr">
-        <is>
-          <t>ノー部活ウィーク</t>
-        </is>
-      </c>
+      <c r="X33" s="211" t="n"/>
       <c r="Y33" s="72" t="n"/>
       <c r="Z33" s="57" t="inlineStr">
         <is>
@@ -10757,7 +10741,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D91"/>
+  <dimension ref="A1:D92"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16.15"/>
   <cols>
     <col width="14" customWidth="1" style="201" min="1" max="1"/>
@@ -12101,37 +12085,44 @@
       </c>
     </row>
     <row r="87">
-      <c r="A87" t="inlineStr">
+      <c r="A87" s="0" t="inlineStr">
         <is>
           <t>・生徒委員会を3/9(木)から3/10(金)へ移動。</t>
         </is>
       </c>
     </row>
     <row r="88">
-      <c r="A88" t="inlineStr">
+      <c r="A88" s="0" t="inlineStr">
         <is>
           <t>・選挙管理委員会・小中連絡会(汐路)を卒業式翌日の3/8(水)へ移動。</t>
         </is>
       </c>
     </row>
     <row r="89">
-      <c r="A89" t="inlineStr">
+      <c r="A89" s="0" t="inlineStr">
         <is>
           <t>・公立一般合格発表(3/6)は日程未定のため赤字。</t>
         </is>
       </c>
     </row>
     <row r="90">
-      <c r="A90" t="inlineStr">
+      <c r="A90" s="0" t="inlineStr">
         <is>
           <t>・2学期期末テストを11/17(水)・11/18(木)へ移動（入学説明会は11/16のまま）。</t>
         </is>
       </c>
     </row>
     <row r="91">
-      <c r="A91" t="inlineStr">
+      <c r="A91" s="0" t="inlineStr">
         <is>
           <t>・学年末テスト(1・2年)を2/17(木)・2/18(金)へ移動。学校保健委員会(学保)も2/17へ移動。2/8・2/9のノー部活デーは残している。</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>・教育相談・保護者会は全学年4日間（木曜を含む）：教育相談5/31〜6/3、保護者会7/5〜7/8、保護者会(3年)・教育相談(1・2年)11/9〜11/12、保護者会12/1〜12/6、保護者会(3年)1/11〜1/14。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add nenkei-sakusei skill and set pre-test no-club weeks in FY2027 plan
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FawjLRytv2ATkyFXeWDDqM
</commit_message>
<xml_diff>
--- a/令和9年度_年間計画（案）.xlsx
+++ b/令和9年度_年間計画（案）.xlsx
@@ -3173,11 +3173,7 @@
       <c r="AF4" s="57" t="n">
         <v>1</v>
       </c>
-      <c r="AG4" s="206" t="inlineStr">
-        <is>
-          <t>ノー部活ウィーク</t>
-        </is>
-      </c>
+      <c r="AG4" s="206" t="n"/>
       <c r="AH4" s="132" t="inlineStr">
         <is>
           <t>▼評</t>
@@ -3229,11 +3225,7 @@
           <t>火</t>
         </is>
       </c>
-      <c r="I5" s="211" t="inlineStr">
-        <is>
-          <t>ノー部活ウィーク</t>
-        </is>
-      </c>
+      <c r="I5" s="211" t="n"/>
       <c r="J5" s="79" t="n"/>
       <c r="K5" s="57" t="inlineStr">
         <is>
@@ -3448,7 +3440,7 @@
       </c>
       <c r="AG6" s="227" t="inlineStr">
         <is>
-          <t>ノー部活ウィーク</t>
+          <t>第２回NCS会議</t>
         </is>
       </c>
       <c r="AH6" s="132" t="n"/>
@@ -3544,11 +3536,7 @@
           <t>水</t>
         </is>
       </c>
-      <c r="I7" s="211" t="inlineStr">
-        <is>
-          <t>ノー部活ウィーク</t>
-        </is>
-      </c>
+      <c r="I7" s="211" t="n"/>
       <c r="J7" s="96" t="n"/>
       <c r="K7" s="57" t="inlineStr">
         <is>
@@ -3612,11 +3600,7 @@
           <t>水</t>
         </is>
       </c>
-      <c r="AG7" s="211" t="inlineStr">
-        <is>
-          <t>第２回NCS会議</t>
-        </is>
-      </c>
+      <c r="AG7" s="211" t="n"/>
       <c r="AH7" s="159" t="n"/>
       <c r="AI7" s="57" t="inlineStr">
         <is>
@@ -3760,7 +3744,7 @@
       </c>
       <c r="AG8" s="206" t="inlineStr">
         <is>
-          <t>ノー部活ウィーク</t>
+          <t>【公立推薦･特色入試】</t>
         </is>
       </c>
       <c r="AH8" s="76" t="inlineStr">
@@ -3854,7 +3838,7 @@
       </c>
       <c r="I9" s="219" t="inlineStr">
         <is>
-          <t>ノー部活ウィーク・歯科健診(IJ･2年午前)・学6(1･3年)</t>
+          <t>歯科健診(IJ･2年午前)・学6(1･3年)</t>
         </is>
       </c>
       <c r="J9" s="157" t="n"/>
@@ -3912,11 +3896,7 @@
           <t>木</t>
         </is>
       </c>
-      <c r="AG9" s="211" t="inlineStr">
-        <is>
-          <t>【公立推薦･特色入試】</t>
-        </is>
-      </c>
+      <c r="AG9" s="211" t="n"/>
       <c r="AH9" s="38" t="inlineStr">
         <is>
           <t>研28</t>
@@ -4010,11 +3990,7 @@
       <c r="H10" s="52" t="n">
         <v>4</v>
       </c>
-      <c r="I10" s="242" t="inlineStr">
-        <is>
-          <t>ノー部活ウィーク</t>
-        </is>
-      </c>
+      <c r="I10" s="242" t="n"/>
       <c r="K10" s="207" t="n">
         <v>4</v>
       </c>
@@ -4057,11 +4033,7 @@
       <c r="AF10" s="52" t="n">
         <v>4</v>
       </c>
-      <c r="AG10" s="206" t="inlineStr">
-        <is>
-          <t>ノー部活ウィーク</t>
-        </is>
-      </c>
+      <c r="AG10" s="206" t="n"/>
       <c r="AH10" s="76" t="n"/>
       <c r="AI10" s="221" t="n">
         <v>4</v>
@@ -4927,7 +4899,7 @@
       </c>
       <c r="AG16" s="206" t="inlineStr">
         <is>
-          <t>ノー部活ウィーク</t>
+          <t>【公立推薦･特色合格発表】</t>
         </is>
       </c>
       <c r="AH16" s="132" t="n"/>
@@ -5090,11 +5062,7 @@
           <t>月</t>
         </is>
       </c>
-      <c r="AG17" s="219" t="inlineStr">
-        <is>
-          <t>【公立推薦･特色合格発表】</t>
-        </is>
-      </c>
+      <c r="AG17" s="219" t="n"/>
       <c r="AH17" s="61" t="n"/>
       <c r="AI17" s="57" t="inlineStr">
         <is>
@@ -5230,11 +5198,7 @@
       <c r="AF18" s="52" t="n">
         <v>8</v>
       </c>
-      <c r="AG18" s="262" t="inlineStr">
-        <is>
-          <t>ノー部活デー</t>
-        </is>
-      </c>
+      <c r="AG18" s="262" t="n"/>
       <c r="AH18" s="144" t="n"/>
       <c r="AI18" s="52" t="n">
         <v>8</v>
@@ -5455,11 +5419,7 @@
       <c r="AF20" s="52" t="n">
         <v>9</v>
       </c>
-      <c r="AG20" s="276" t="inlineStr">
-        <is>
-          <t>ノー部活デー</t>
-        </is>
-      </c>
+      <c r="AG20" s="276" t="n"/>
       <c r="AH20" s="141" t="n"/>
       <c r="AI20" s="52" t="n">
         <v>9</v>
@@ -5552,7 +5512,7 @@
       </c>
       <c r="X21" s="136" t="inlineStr">
         <is>
-          <t>教育相談(1・2年)・ノー部活ウィーク</t>
+          <t>教育相談(1・2年)</t>
         </is>
       </c>
       <c r="Y21" s="85" t="n"/>
@@ -5682,7 +5642,11 @@
       <c r="AF22" s="52" t="n">
         <v>10</v>
       </c>
-      <c r="AG22" s="206" t="n"/>
+      <c r="AG22" s="206" t="inlineStr">
+        <is>
+          <t>ノー部活ウィーク</t>
+        </is>
+      </c>
       <c r="AH22" s="76" t="inlineStr">
         <is>
           <t>全反</t>
@@ -6602,7 +6566,11 @@
           <t>月</t>
         </is>
       </c>
-      <c r="AG31" s="18" t="n"/>
+      <c r="AG31" s="18" t="inlineStr">
+        <is>
+          <t>ノー部活ウィーク</t>
+        </is>
+      </c>
       <c r="AH31" s="38" t="inlineStr">
         <is>
           <t>委</t>
@@ -6825,7 +6793,11 @@
           <t>火</t>
         </is>
       </c>
-      <c r="AG33" s="18" t="n"/>
+      <c r="AG33" s="18" t="inlineStr">
+        <is>
+          <t>ノー部活ウィーク</t>
+        </is>
+      </c>
       <c r="AH33" s="95" t="n"/>
       <c r="AI33" s="57" t="inlineStr">
         <is>
@@ -7013,7 +6985,11 @@
           <t>火</t>
         </is>
       </c>
-      <c r="X35" s="219" t="n"/>
+      <c r="X35" s="219" t="inlineStr">
+        <is>
+          <t>ノー部活ウィーク</t>
+        </is>
+      </c>
       <c r="Y35" s="38" t="n"/>
       <c r="Z35" s="57" t="inlineStr">
         <is>
@@ -7039,7 +7015,11 @@
           <t>水</t>
         </is>
       </c>
-      <c r="AG35" s="321" t="n"/>
+      <c r="AG35" s="321" t="inlineStr">
+        <is>
+          <t>ノー部活ウィーク</t>
+        </is>
+      </c>
       <c r="AI35" s="57" t="inlineStr">
         <is>
           <t>木</t>
@@ -7182,7 +7162,11 @@
           <t>木</t>
         </is>
       </c>
-      <c r="I37" s="70" t="n"/>
+      <c r="I37" s="70" t="inlineStr">
+        <is>
+          <t>ノー部活ウィーク</t>
+        </is>
+      </c>
       <c r="J37" s="61" t="inlineStr">
         <is>
           <t>運6
@@ -7386,7 +7370,11 @@
           <t>金</t>
         </is>
       </c>
-      <c r="I39" s="115" t="n"/>
+      <c r="I39" s="115" t="inlineStr">
+        <is>
+          <t>ノー部活ウィーク</t>
+        </is>
+      </c>
       <c r="J39" s="111" t="n"/>
       <c r="K39" s="203" t="inlineStr">
         <is>
@@ -7895,7 +7883,11 @@
       <c r="H44" s="65" t="n">
         <v>21</v>
       </c>
-      <c r="I44" s="16" t="n"/>
+      <c r="I44" s="16" t="inlineStr">
+        <is>
+          <t>ノー部活ウィーク</t>
+        </is>
+      </c>
       <c r="J44" s="147" t="n"/>
       <c r="K44" s="52" t="n">
         <v>21</v>
@@ -8171,7 +8163,11 @@
           <t>火</t>
         </is>
       </c>
-      <c r="I47" s="18" t="n"/>
+      <c r="I47" s="18" t="inlineStr">
+        <is>
+          <t>ノー部活ウィーク</t>
+        </is>
+      </c>
       <c r="J47" s="38" t="n"/>
       <c r="K47" s="57" t="inlineStr">
         <is>
@@ -8263,7 +8259,11 @@
       <c r="H48" s="97" t="n">
         <v>23</v>
       </c>
-      <c r="I48" s="14" t="n"/>
+      <c r="I48" s="14" t="inlineStr">
+        <is>
+          <t>ノー部活ウィーク</t>
+        </is>
+      </c>
       <c r="J48" s="104" t="n"/>
       <c r="K48" s="52" t="n">
         <v>23</v>
@@ -8487,7 +8487,7 @@
       </c>
       <c r="R50" s="234" t="inlineStr">
         <is>
-          <t>ノー部活ウィーク</t>
+          <t>専修合同説明会</t>
         </is>
       </c>
       <c r="S50" s="103" t="inlineStr">
@@ -8600,7 +8600,7 @@
       </c>
       <c r="R51" s="346" t="inlineStr">
         <is>
-          <t>専修合同説明会</t>
+          <t>ノー部活ウィーク</t>
         </is>
       </c>
       <c r="S51" s="92" t="n"/>
@@ -10004,11 +10004,7 @@
           <t>月</t>
         </is>
       </c>
-      <c r="F65" s="44" t="inlineStr">
-        <is>
-          <t>ノー部活ウィーク</t>
-        </is>
-      </c>
+      <c r="F65" s="44" t="n"/>
       <c r="G65" s="43" t="n"/>
       <c r="K65" s="366" t="inlineStr">
         <is>
@@ -10741,7 +10737,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D92"/>
+  <dimension ref="A1:D93"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16.15"/>
   <cols>
     <col width="14" customWidth="1" style="201" min="1" max="1"/>
@@ -12120,9 +12116,16 @@
       </c>
     </row>
     <row r="92">
-      <c r="A92" t="inlineStr">
+      <c r="A92" s="0" t="inlineStr">
         <is>
           <t>・教育相談・保護者会は全学年4日間（木曜を含む）：教育相談5/31〜6/3、保護者会7/5〜7/8、保護者会(3年)・教育相談(1・2年)11/9〜11/12、保護者会12/1〜12/6、保護者会(3年)1/11〜1/14。</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>・ノー部活ウィークはテスト前1週間（6/17〜6/23、9/21〜9/24、11/10〜11/16、2/10〜2/16）。夏季・冬季の閉庁期間のものは残した。2/8・2/9のノー部活デーは学年末テストの移動に合わせて削除。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Move grade 1 parents' meeting to 2/25
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FawjLRytv2ATkyFXeWDDqM
</commit_message>
<xml_diff>
--- a/令和9年度_年間計画（案）.xlsx
+++ b/令和9年度_年間計画（案）.xlsx
@@ -7229,7 +7229,7 @@
       </c>
       <c r="AG37" s="276" t="inlineStr">
         <is>
-          <t>学年保護者会(1年)・【定時制合格発表】</t>
+          <t>【定時制合格発表】</t>
         </is>
       </c>
       <c r="AH37" s="61" t="inlineStr">
@@ -8841,7 +8841,7 @@
       </c>
       <c r="AG53" s="13" t="inlineStr">
         <is>
-          <t>【公立一般Ｂ面接】</t>
+          <t>【公立一般Ｂ面接】・学年保護者会(1年)</t>
         </is>
       </c>
       <c r="AH53" s="61" t="n"/>
@@ -10737,7 +10737,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D93"/>
+  <dimension ref="A1:D94"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16.15"/>
   <cols>
     <col width="14" customWidth="1" style="201" min="1" max="1"/>
@@ -12123,9 +12123,16 @@
       </c>
     </row>
     <row r="93">
-      <c r="A93" t="inlineStr">
+      <c r="A93" s="0" t="inlineStr">
         <is>
           <t>・ノー部活ウィークはテスト前1週間（6/17〜6/23、9/21〜9/24、11/10〜11/16、2/10〜2/16）。夏季・冬季の閉庁期間のものは残した。2/8・2/9のノー部活デーは学年末テストの移動に合わせて削除。</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>・学年保護者会(1年)を2/17(学年末テスト)から2/25(金)へ移動。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Move grade 1 parents' meeting to 2/22
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FawjLRytv2ATkyFXeWDDqM
</commit_message>
<xml_diff>
--- a/令和9年度_年間計画（案）.xlsx
+++ b/令和9年度_年間計画（案）.xlsx
@@ -8127,7 +8127,11 @@
       <c r="AF46" s="52" t="n">
         <v>22</v>
       </c>
-      <c r="AG46" s="64" t="n"/>
+      <c r="AG46" s="64" t="inlineStr">
+        <is>
+          <t>学年保護者会(1年)</t>
+        </is>
+      </c>
       <c r="AH46" s="101" t="n"/>
       <c r="AI46" s="52" t="n">
         <v>22</v>
@@ -8841,7 +8845,7 @@
       </c>
       <c r="AG53" s="13" t="inlineStr">
         <is>
-          <t>【公立一般Ｂ面接】・学年保護者会(1年)</t>
+          <t>【公立一般Ｂ面接】</t>
         </is>
       </c>
       <c r="AH53" s="61" t="n"/>
@@ -10737,7 +10741,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D94"/>
+  <dimension ref="A1:D95"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16.15"/>
   <cols>
     <col width="14" customWidth="1" style="201" min="1" max="1"/>
@@ -12130,9 +12134,16 @@
       </c>
     </row>
     <row r="94">
-      <c r="A94" t="inlineStr">
+      <c r="A94" s="0" t="inlineStr">
         <is>
           <t>・学年保護者会(1年)を2/17(学年末テスト)から2/25(金)へ移動。</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>・学年保護者会(1年)は3送会リハと重ならないよう2/22(火)へ（2/25から再移動）。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Export FY2027 annual plan PDF for review
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FawjLRytv2ATkyFXeWDDqM
</commit_message>
<xml_diff>
--- a/令和9年度_年間計画（案）.xlsx
+++ b/令和9年度_年間計画（案）.xlsx
@@ -1194,7 +1194,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="31" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="429">
+  <cellXfs count="431">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <protection locked="0" hidden="0"/>
     </xf>
@@ -2428,6 +2428,12 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="1" fontId="35" fillId="0" borderId="26" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="2">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="33" fillId="0" borderId="66" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="2">
+      <alignment vertical="center" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="33" fillId="0" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="2">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -6566,7 +6572,7 @@
           <t>月</t>
         </is>
       </c>
-      <c r="AG31" s="18" t="inlineStr">
+      <c r="AG31" s="414" t="inlineStr">
         <is>
           <t>ノー部活ウィーク</t>
         </is>
@@ -6793,7 +6799,7 @@
           <t>火</t>
         </is>
       </c>
-      <c r="AG33" s="18" t="inlineStr">
+      <c r="AG33" s="414" t="inlineStr">
         <is>
           <t>ノー部活ウィーク</t>
         </is>
@@ -7015,7 +7021,7 @@
           <t>水</t>
         </is>
       </c>
-      <c r="AG35" s="321" t="inlineStr">
+      <c r="AG35" s="429" t="inlineStr">
         <is>
           <t>ノー部活ウィーク</t>
         </is>
@@ -7162,7 +7168,7 @@
           <t>木</t>
         </is>
       </c>
-      <c r="I37" s="70" t="inlineStr">
+      <c r="I37" s="430" t="inlineStr">
         <is>
           <t>ノー部活ウィーク</t>
         </is>
@@ -7370,7 +7376,7 @@
           <t>金</t>
         </is>
       </c>
-      <c r="I39" s="115" t="inlineStr">
+      <c r="I39" s="419" t="inlineStr">
         <is>
           <t>ノー部活ウィーク</t>
         </is>
@@ -7883,7 +7889,7 @@
       <c r="H44" s="65" t="n">
         <v>21</v>
       </c>
-      <c r="I44" s="16" t="inlineStr">
+      <c r="I44" s="413" t="inlineStr">
         <is>
           <t>ノー部活ウィーク</t>
         </is>
@@ -7906,7 +7912,7 @@
       <c r="Q44" s="65" t="n">
         <v>21</v>
       </c>
-      <c r="R44" s="245" t="inlineStr">
+      <c r="R44" s="424" t="inlineStr">
         <is>
           <t>ノー部活ウィーク</t>
         </is>
@@ -8167,7 +8173,7 @@
           <t>火</t>
         </is>
       </c>
-      <c r="I47" s="18" t="inlineStr">
+      <c r="I47" s="414" t="inlineStr">
         <is>
           <t>ノー部活ウィーク</t>
         </is>
@@ -8263,7 +8269,7 @@
       <c r="H48" s="97" t="n">
         <v>23</v>
       </c>
-      <c r="I48" s="14" t="inlineStr">
+      <c r="I48" s="416" t="inlineStr">
         <is>
           <t>ノー部活ウィーク</t>
         </is>
@@ -9824,7 +9830,7 @@
       <c r="Z64" s="52" t="n">
         <v>31</v>
       </c>
-      <c r="AA64" s="22" t="inlineStr">
+      <c r="AA64" s="423" t="inlineStr">
         <is>
           <t>ノー部活ウィーク</t>
         </is>
@@ -12141,7 +12147,7 @@
       </c>
     </row>
     <row r="95">
-      <c r="A95" t="inlineStr">
+      <c r="A95" s="0" t="inlineStr">
         <is>
           <t>・学年保護者会(1年)は3送会リハと重ならないよう2/22(火)へ（2/25から再移動）。</t>
         </is>

</xml_diff>

<commit_message>
Add grade 3 home study day on 6/11
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FawjLRytv2ATkyFXeWDDqM
</commit_message>
<xml_diff>
--- a/令和9年度_年間計画（案）.xlsx
+++ b/令和9年度_年間計画（案）.xlsx
@@ -3863,7 +3863,7 @@
           <t>８　月</t>
         </is>
       </c>
-      <c r="O3" s="437" t="n"/>
+      <c r="O3" s="546" t="n"/>
       <c r="P3" s="433" t="n"/>
       <c r="Q3" s="435" t="n"/>
       <c r="R3" s="432" t="inlineStr">
@@ -6627,7 +6627,11 @@
       <c r="H24" s="463" t="n">
         <v>11</v>
       </c>
-      <c r="I24" s="490" t="n"/>
+      <c r="I24" s="490" t="inlineStr">
+        <is>
+          <t>家庭学習日(3年)</t>
+        </is>
+      </c>
       <c r="J24" s="630" t="inlineStr">
         <is>
           <t>定</t>
@@ -11607,7 +11611,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D95"/>
+  <dimension ref="A1:D96"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16.15"/>
   <cols>
     <col width="14" customWidth="1" style="201" min="1" max="1"/>
@@ -13013,6 +13017,13 @@
         </is>
       </c>
     </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>・6/11(金)を家庭学習日(3年)とした（修学旅行の翌日）。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Schedule learning-frame sessions (Thu 50min + Mon/Wed 25min) in FY2027 plan
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FawjLRytv2ATkyFXeWDDqM
</commit_message>
<xml_diff>
--- a/令和9年度_年間計画（案）.xlsx
+++ b/令和9年度_年間計画（案）.xlsx
@@ -3858,7 +3858,7 @@
         </is>
       </c>
       <c r="M3" s="433" t="n"/>
-      <c r="N3" s="436" t="inlineStr">
+      <c r="N3" s="584" t="inlineStr">
         <is>
           <t>８　月</t>
         </is>
@@ -3991,7 +3991,11 @@
         <v>1</v>
       </c>
       <c r="X4" s="448" t="n"/>
-      <c r="Y4" s="622" t="n"/>
+      <c r="Y4" s="622" t="inlineStr">
+        <is>
+          <t>探½</t>
+        </is>
+      </c>
       <c r="Z4" s="438" t="n">
         <v>1</v>
       </c>
@@ -4076,7 +4080,8 @@
       <c r="M5" s="629" t="inlineStr">
         <is>
           <t>職6
-研10</t>
+研10
+探9</t>
         </is>
       </c>
       <c r="N5" s="455" t="inlineStr">
@@ -4401,7 +4406,8 @@
       <c r="S7" s="629" t="inlineStr">
         <is>
           <t>現4
-研12</t>
+研12
+探11</t>
         </is>
       </c>
       <c r="T7" s="455" t="inlineStr">
@@ -4449,7 +4455,11 @@
         </is>
       </c>
       <c r="AJ7" s="460" t="n"/>
-      <c r="AK7" s="626" t="n"/>
+      <c r="AK7" s="626" t="inlineStr">
+        <is>
+          <t>探24</t>
+        </is>
+      </c>
       <c r="AL7" s="450" t="n"/>
       <c r="AM7" s="451" t="n"/>
       <c r="AN7" s="152" t="inlineStr">
@@ -4744,7 +4754,8 @@
       <c r="AG9" s="458" t="n"/>
       <c r="AH9" s="626" t="inlineStr">
         <is>
-          <t>研28</t>
+          <t>研28
+探21</t>
         </is>
       </c>
       <c r="AI9" s="452" t="inlineStr">
@@ -4852,7 +4863,11 @@
         <v>4</v>
       </c>
       <c r="U10" s="472" t="n"/>
-      <c r="V10" s="630" t="n"/>
+      <c r="V10" s="630" t="inlineStr">
+        <is>
+          <t>探½</t>
+        </is>
+      </c>
       <c r="W10" s="463" t="n">
         <v>4</v>
       </c>
@@ -5509,7 +5524,8 @@
       <c r="F15" s="492" t="n"/>
       <c r="G15" s="626" t="inlineStr">
         <is>
-          <t>研4</t>
+          <t>研4
+探4</t>
         </is>
       </c>
       <c r="H15" s="455" t="inlineStr">
@@ -5834,7 +5850,11 @@
         </is>
       </c>
       <c r="I17" s="460" t="n"/>
-      <c r="J17" s="626" t="n"/>
+      <c r="J17" s="626" t="inlineStr">
+        <is>
+          <t>探½</t>
+        </is>
+      </c>
       <c r="K17" s="452" t="inlineStr">
         <is>
           <t>水</t>
@@ -6023,7 +6043,11 @@
         <v>8</v>
       </c>
       <c r="X18" s="471" t="n"/>
-      <c r="Y18" s="630" t="n"/>
+      <c r="Y18" s="630" t="inlineStr">
+        <is>
+          <t>探½</t>
+        </is>
+      </c>
       <c r="Z18" s="463" t="n">
         <v>8</v>
       </c>
@@ -6047,7 +6071,11 @@
           <t>選挙管理委員会</t>
         </is>
       </c>
-      <c r="AK18" s="630" t="n"/>
+      <c r="AK18" s="630" t="inlineStr">
+        <is>
+          <t>探½</t>
+        </is>
+      </c>
       <c r="AL18" s="450" t="n"/>
       <c r="AM18" s="451" t="n"/>
       <c r="AO18" s="3">
@@ -6089,7 +6117,8 @@
           <t>努･採
 運2
 職2
-研1</t>
+研1
+探1</t>
         </is>
       </c>
       <c r="E19" s="455" t="inlineStr">
@@ -6228,7 +6257,11 @@
           <t>私立合同説明会</t>
         </is>
       </c>
-      <c r="S20" s="630" t="n"/>
+      <c r="S20" s="630" t="inlineStr">
+        <is>
+          <t>探12</t>
+        </is>
+      </c>
       <c r="T20" s="466" t="n">
         <v>9</v>
       </c>
@@ -6366,7 +6399,8 @@
       <c r="AB21" s="629" t="inlineStr">
         <is>
           <t>進4
-研22</t>
+研22
+探18</t>
         </is>
       </c>
       <c r="AC21" s="455" t="inlineStr">
@@ -6594,7 +6628,8 @@
       <c r="AG23" s="499" t="n"/>
       <c r="AH23" s="626" t="inlineStr">
         <is>
-          <t>研29</t>
+          <t>研29
+探22</t>
         </is>
       </c>
       <c r="AI23" s="452" t="inlineStr">
@@ -6818,7 +6853,11 @@
           <t>身体測定(2年)</t>
         </is>
       </c>
-      <c r="D26" s="630" t="n"/>
+      <c r="D26" s="630" t="inlineStr">
+        <is>
+          <t>探½</t>
+        </is>
+      </c>
       <c r="E26" s="463" t="n">
         <v>12</v>
       </c>
@@ -7136,7 +7175,8 @@
       <c r="G29" s="629" t="inlineStr">
         <is>
           <t>職4
-研5</t>
+研5
+探5</t>
         </is>
       </c>
       <c r="H29" s="455" t="inlineStr">
@@ -7231,7 +7271,11 @@
           <t>身体測定(欠席者)</t>
         </is>
       </c>
-      <c r="D30" s="630" t="n"/>
+      <c r="D30" s="630" t="inlineStr">
+        <is>
+          <t>探½</t>
+        </is>
+      </c>
       <c r="E30" s="463" t="n">
         <v>14</v>
       </c>
@@ -7305,7 +7349,11 @@
           <t>※【定時制１次入試】</t>
         </is>
       </c>
-      <c r="AH30" s="630" t="n"/>
+      <c r="AH30" s="630" t="inlineStr">
+        <is>
+          <t>探½</t>
+        </is>
+      </c>
       <c r="AI30" s="463" t="n">
         <v>14</v>
       </c>
@@ -7379,7 +7427,8 @@
       <c r="U31" s="460" t="n"/>
       <c r="V31" s="626" t="inlineStr">
         <is>
-          <t>研16</t>
+          <t>研16
+探14</t>
         </is>
       </c>
       <c r="W31" s="455" t="inlineStr">
@@ -7505,7 +7554,11 @@
           <t>ノー部活ウィーク</t>
         </is>
       </c>
-      <c r="Y32" s="630" t="n"/>
+      <c r="Y32" s="630" t="inlineStr">
+        <is>
+          <t>探½</t>
+        </is>
+      </c>
       <c r="Z32" s="463" t="n">
         <v>15</v>
       </c>
@@ -7560,7 +7613,8 @@
           <t>運3
 不
 進1
-研2</t>
+研2
+探2</t>
         </is>
       </c>
       <c r="E33" s="455" t="inlineStr">
@@ -7587,7 +7641,11 @@
           <t>小中努力点交流会</t>
         </is>
       </c>
-      <c r="M33" s="626" t="n"/>
+      <c r="M33" s="626" t="inlineStr">
+        <is>
+          <t>探10</t>
+        </is>
+      </c>
       <c r="N33" s="455" t="inlineStr">
         <is>
           <t>日</t>
@@ -7748,7 +7806,11 @@
           <t>【公立一般志願変更】</t>
         </is>
       </c>
-      <c r="AH34" s="630" t="n"/>
+      <c r="AH34" s="630" t="inlineStr">
+        <is>
+          <t>探½</t>
+        </is>
+      </c>
       <c r="AI34" s="463" t="n">
         <v>16</v>
       </c>
@@ -7816,7 +7878,8 @@
       <c r="S35" s="629" t="inlineStr">
         <is>
           <t>教
-研14</t>
+研14
+探13</t>
         </is>
       </c>
       <c r="T35" s="455" t="inlineStr">
@@ -7845,7 +7908,8 @@
       <c r="AA35" s="453" t="n"/>
       <c r="AB35" s="626" t="inlineStr">
         <is>
-          <t>研23</t>
+          <t>研23
+探19</t>
         </is>
       </c>
       <c r="AC35" s="455" t="inlineStr">
@@ -7875,7 +7939,8 @@
       <c r="AK35" s="648" t="inlineStr">
         <is>
           <t>採
-研34</t>
+研34
+探25</t>
         </is>
       </c>
       <c r="AL35" s="450" t="n"/>
@@ -7962,7 +8027,11 @@
         <v>17</v>
       </c>
       <c r="AD36" s="471" t="n"/>
-      <c r="AE36" s="630" t="n"/>
+      <c r="AE36" s="630" t="inlineStr">
+        <is>
+          <t>探½</t>
+        </is>
+      </c>
       <c r="AF36" s="463" t="n">
         <v>17</v>
       </c>
@@ -8015,7 +8084,8 @@
       <c r="J37" s="629" t="inlineStr">
         <is>
           <t>運6
-研8</t>
+研8
+探8</t>
         </is>
       </c>
       <c r="K37" s="455" t="inlineStr">
@@ -8413,7 +8483,8 @@
       <c r="C41" s="453" t="n"/>
       <c r="D41" s="626" t="inlineStr">
         <is>
-          <t>委</t>
+          <t>委
+探½</t>
         </is>
       </c>
       <c r="E41" s="452" t="inlineStr">
@@ -8579,7 +8650,11 @@
         <v>20</v>
       </c>
       <c r="AA42" s="471" t="n"/>
-      <c r="AB42" s="630" t="n"/>
+      <c r="AB42" s="630" t="inlineStr">
+        <is>
+          <t>探½</t>
+        </is>
+      </c>
       <c r="AC42" s="463" t="n">
         <v>20</v>
       </c>
@@ -8629,7 +8704,8 @@
       <c r="G43" s="629" t="inlineStr">
         <is>
           <t>現2
-研6</t>
+研6
+探6</t>
         </is>
       </c>
       <c r="H43" s="455" t="inlineStr">
@@ -8720,7 +8796,11 @@
         <v>21</v>
       </c>
       <c r="C44" s="490" t="n"/>
-      <c r="D44" s="630" t="n"/>
+      <c r="D44" s="630" t="inlineStr">
+        <is>
+          <t>探½</t>
+        </is>
+      </c>
       <c r="E44" s="463" t="n">
         <v>21</v>
       </c>
@@ -8734,7 +8814,11 @@
           <t>ノー部活ウィーク</t>
         </is>
       </c>
-      <c r="J44" s="630" t="n"/>
+      <c r="J44" s="630" t="inlineStr">
+        <is>
+          <t>探½</t>
+        </is>
+      </c>
       <c r="K44" s="463" t="n">
         <v>21</v>
       </c>
@@ -8850,7 +8934,11 @@
         </is>
       </c>
       <c r="U45" s="460" t="n"/>
-      <c r="V45" s="626" t="n"/>
+      <c r="V45" s="626" t="inlineStr">
+        <is>
+          <t>探15</t>
+        </is>
+      </c>
       <c r="W45" s="455" t="inlineStr">
         <is>
           <t>日</t>
@@ -8983,7 +9071,11 @@
         <v>22</v>
       </c>
       <c r="AJ46" s="471" t="n"/>
-      <c r="AK46" s="630" t="n"/>
+      <c r="AK46" s="630" t="inlineStr">
+        <is>
+          <t>探½</t>
+        </is>
+      </c>
       <c r="AL46" s="450" t="n"/>
       <c r="AM46" s="451" t="n"/>
       <c r="BA46" s="377" t="n"/>
@@ -8998,7 +9090,8 @@
       <c r="C47" s="460" t="n"/>
       <c r="D47" s="626" t="inlineStr">
         <is>
-          <t>研3</t>
+          <t>研3
+探3</t>
         </is>
       </c>
       <c r="E47" s="455" t="inlineStr">
@@ -9114,7 +9207,11 @@
           <t>ノー部活ウィーク</t>
         </is>
       </c>
-      <c r="J48" s="632" t="n"/>
+      <c r="J48" s="632" t="inlineStr">
+        <is>
+          <t>探½</t>
+        </is>
+      </c>
       <c r="K48" s="463" t="n">
         <v>23</v>
       </c>
@@ -9496,7 +9593,8 @@
       <c r="AH51" s="629" t="inlineStr">
         <is>
           <t>教
-研31</t>
+研31
+探23</t>
         </is>
       </c>
       <c r="AI51" s="452" t="inlineStr">
@@ -9667,7 +9765,8 @@
       <c r="Y53" s="648" t="inlineStr">
         <is>
           <t>学10
-研21</t>
+研21
+探17</t>
         </is>
       </c>
       <c r="Z53" s="455" t="inlineStr">
@@ -10001,7 +10100,8 @@
       </c>
       <c r="G57" s="626" t="inlineStr">
         <is>
-          <t>研7</t>
+          <t>研7
+探7</t>
         </is>
       </c>
       <c r="H57" s="455" t="inlineStr">
@@ -10065,7 +10165,8 @@
       <c r="AD57" s="499" t="n"/>
       <c r="AE57" s="626" t="inlineStr">
         <is>
-          <t>研27</t>
+          <t>研27
+探20</t>
         </is>
       </c>
       <c r="AF57" s="455" t="inlineStr">
@@ -10091,7 +10192,11 @@
         <v>28</v>
       </c>
       <c r="C58" s="497" t="n"/>
-      <c r="D58" s="630" t="n"/>
+      <c r="D58" s="630" t="inlineStr">
+        <is>
+          <t>探½</t>
+        </is>
+      </c>
       <c r="E58" s="463" t="n">
         <v>28</v>
       </c>
@@ -10230,7 +10335,8 @@
       <c r="U59" s="460" t="n"/>
       <c r="V59" s="626" t="inlineStr">
         <is>
-          <t>研18</t>
+          <t>研18
+探16</t>
         </is>
       </c>
       <c r="W59" s="455" t="inlineStr">
@@ -10314,7 +10420,11 @@
           <t>体育大会係生徒打合せ</t>
         </is>
       </c>
-      <c r="S60" s="630" t="n"/>
+      <c r="S60" s="630" t="inlineStr">
+        <is>
+          <t>探½</t>
+        </is>
+      </c>
       <c r="T60" s="463" t="n">
         <v>29</v>
       </c>
@@ -10421,7 +10531,11 @@
         </is>
       </c>
       <c r="X61" s="460" t="n"/>
-      <c r="Y61" s="626" t="n"/>
+      <c r="Y61" s="626" t="inlineStr">
+        <is>
+          <t>探½</t>
+        </is>
+      </c>
       <c r="Z61" s="452" t="inlineStr">
         <is>
           <t>水</t>
@@ -11611,7 +11725,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D96"/>
+  <dimension ref="A1:D98"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16.15"/>
   <cols>
     <col width="14" customWidth="1" style="201" min="1" max="1"/>
@@ -13018,9 +13132,23 @@
       </c>
     </row>
     <row r="96">
-      <c r="A96" t="inlineStr">
+      <c r="A96" s="0" t="inlineStr">
         <is>
           <t>・6/11(金)を家庭学習日(3年)とした（修学旅行の翌日）。</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>・学習枠：木曜5限後13:50〜14:40（50分）を25回（会議記号の列「探1〜」）。木曜が使えない週は月・水の6限後14:45〜15:10（25分）を20回（「探½」）。合計35時数。</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>・木曜の流れ：5限→学習枠13:50〜14:40→短学→14:50下校→研修14:55〜15:45（会議は研修の中で行う）。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add one period on cleanup days to secure grade 1 hours
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FawjLRytv2ATkyFXeWDDqM
</commit_message>
<xml_diff>
--- a/令和9年度_年間計画（案）.xlsx
+++ b/令和9年度_年間計画（案）.xlsx
@@ -11725,7 +11725,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D98"/>
+  <dimension ref="A1:D99"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16.15"/>
   <cols>
     <col width="14" customWidth="1" style="201" min="1" max="1"/>
@@ -13139,16 +13139,23 @@
       </c>
     </row>
     <row r="97">
-      <c r="A97" t="inlineStr">
+      <c r="A97" s="0" t="inlineStr">
         <is>
           <t>・学習枠：木曜5限後13:50〜14:40（50分）を25回（会議記号の列「探1〜」）。木曜が使えない週は月・水の6限後14:45〜15:10（25分）を20回（「探½」）。合計35時数。</t>
         </is>
       </c>
     </row>
     <row r="98">
-      <c r="A98" t="inlineStr">
+      <c r="A98" s="0" t="inlineStr">
         <is>
           <t>・木曜の流れ：5限→学習枠13:50〜14:40→短学→14:50下校→研修14:55〜15:45（会議は研修の中で行う）。</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>・大掃除の日（7/16・12/22・3/23）は授業を1コマ増やす（1年の時数確保のため）。テストの日の午後と4月初めは授業を増やさない。</t>
         </is>
       </c>
     </row>

</xml_diff>